<commit_message>
fix: recover a 7/27 MLB pick lost from main ledger by the clear/recreate bug
Seattle Mariners @ Texas Rangers (event 401816288, 2026-07-27) was a real,
genuinely qualified pregame call that a daily re-forecast cycle cleared from
picks.xlsx and then failed to recreate (same class of bug fixed in ledger.py
this session). The row survived intact, fully settled, in flat_picks.xlsx
with its original pregame decision timestamps.

Restored via PickLedger.import_rows -- the ledger's own sanctioned path for
re-adding an already-existing immutable record without fabricating a new
decision timestamp, distinct from creating a fresh pick (which correctly
refuses once an event has started). Audit chain records the recovery and
its reason plainly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO22" headerRowCount="1">
-  <autoFilter ref="A1:CO22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO21" headerRowCount="1">
+  <autoFilter ref="A1:CO21"/>
   <tableColumns count="93">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -752,19 +752,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$22)</f>
+        <f>COUNTA('Picks'!$A$2:$A$21)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$22,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$21,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$22,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"win")+COUNTIFS('Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")+COUNTIFS('Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -792,19 +792,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$22,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$21,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$22,"&gt;0",'Picks'!$V$2:$V$22,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$22,"&gt;0",'Picks'!$V$2:$V$22,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$22,"&gt;0",'Picks'!$V$2:$V$22,"win")/(COUNTIFS('Picks'!$BX$2:$BX$22,"&gt;0",'Picks'!$V$2:$V$22,"win")+COUNTIFS('Picks'!$BX$2:$BX$22,"&gt;0",'Picks'!$V$2:$V$22,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"win")/(COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"win")+COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$22)/SUM('Picks'!$BX$2:$BX$22),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$21)/SUM('Picks'!$BX$2:$BX$21),0)</f>
         <v/>
       </c>
     </row>
@@ -832,19 +832,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$22)</f>
+        <f>SUM('Picks'!$BY$2:$BY$21)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$22,"&lt;&gt;",'Picks'!$AB$2:$AB$22),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$21,"&lt;&gt;",'Picks'!$AB$2:$AB$21),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$22,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$22,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$21,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$22,'Picks'!$AM$2:$AM$22,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$21,'Picks'!$AM$2:$AM$21,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -899,15 +899,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A14,'Picks'!$U$2:$U$22,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A14,'Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A14,'Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -915,11 +915,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$22,'Picks'!$H$2:$H$22,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$21,'Picks'!$H$2:$H$21,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$22,'Picks'!$H$2:$H$22,$A14,'Picks'!$U$2:$U$22,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$21,'Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -930,15 +930,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A15,'Picks'!$U$2:$U$22,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A15,'Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A15,'Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -946,11 +946,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$22,'Picks'!$H$2:$H$22,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$21,'Picks'!$H$2:$H$21,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$22,'Picks'!$H$2:$H$22,$A15,'Picks'!$U$2:$U$22,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$21,'Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -961,15 +961,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A16,'Picks'!$U$2:$U$22,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A16,'Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$22,$A16,'Picks'!$U$2:$U$22,"settled",'Picks'!$V$2:$V$22,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -977,11 +977,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$22,'Picks'!$H$2:$H$22,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$21,'Picks'!$H$2:$H$21,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$22,'Picks'!$H$2:$H$22,$A16,'Picks'!$U$2:$U$22,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$21,'Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CO22"/>
+  <dimension ref="A1:CO21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5153,12 +5153,12 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>7681c20815f547e4</t>
+          <t>b130a7489baa41ec</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T05:05:50.168792Z</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
@@ -5231,18 +5231,32 @@
       </c>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V15" s="24" t="n"/>
-      <c r="W15" s="26" t="n"/>
-      <c r="X15" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W15" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y15" s="25" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n"/>
-      <c r="AD15" s="24" t="n"/>
+      <c r="AC15" s="30" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AD15" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T11:12:40.671751Z</t>
+        </is>
+      </c>
       <c r="AE15" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.4600 (market_slug=aec-cs2-bpl-enjoy-2026-07-28).</t>
@@ -5255,7 +5269,7 @@
       </c>
       <c r="AG15" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH15" s="24" t="n"/>
@@ -5329,7 +5343,7 @@
       </c>
       <c r="BA15" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>40c2937bc668bb862cf7af94b4e50bd7f49459da4b5b52e8a268f7bbef6d0377</t>
         </is>
       </c>
       <c r="BB15" s="24" t="inlineStr">
@@ -5344,7 +5358,7 @@
       </c>
       <c r="BD15" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>40c2937bc668bb862cf7af94b4e50bd7f49459da4b5b52e8a268f7bbef6d0377</t>
         </is>
       </c>
       <c r="BE15" s="24" t="inlineStr">
@@ -5364,7 +5378,7 @@
       </c>
       <c r="BH15" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:39.784703Z</t>
+          <t>2026-07-28T05:05:25.710714Z</t>
         </is>
       </c>
       <c r="BI15" s="24" t="inlineStr">
@@ -5414,22 +5428,22 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>6a4e6e1f199546c9</t>
+          <t>b3a9bdbbf6b748de</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T05:05:50.168792Z</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T10:00:00Z</t>
+          <t>2026-07-28T08:00:00Z</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>64432</t>
+          <t>63706</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
@@ -5439,12 +5453,12 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>MOUZ NXT</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
-          <t>Noir Verse</t>
+          <t>Entropy</t>
         </is>
       </c>
       <c r="H16" s="24" t="inlineStr">
@@ -5464,26 +5478,26 @@
         </is>
       </c>
       <c r="L16" s="26" t="n">
-        <v>186</v>
+        <v>-144</v>
       </c>
       <c r="M16" s="27" t="n">
-        <v>2.86</v>
+        <v>1.694444</v>
       </c>
       <c r="N16" s="28" t="n">
-        <v>0.34965</v>
+        <v>0.590164</v>
       </c>
       <c r="O16" s="28" t="n">
-        <v>0.509533</v>
+        <v>0.609287</v>
       </c>
       <c r="P16" s="28" t="n"/>
       <c r="Q16" s="28" t="n">
-        <v>0.159883</v>
+        <v>0.019123</v>
       </c>
       <c r="R16" s="26" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="S16" s="29" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="T16" s="24" t="inlineStr">
         <is>
@@ -5492,21 +5506,35 @@
       </c>
       <c r="U16" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V16" s="24" t="n"/>
-      <c r="W16" s="26" t="n"/>
-      <c r="X16" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V16" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W16" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y16" s="25" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="30" t="n"/>
-      <c r="AD16" s="24" t="n"/>
+      <c r="AC16" s="30" t="n">
+        <v>1.0417</v>
+      </c>
+      <c r="AD16" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T11:12:41.886189Z</t>
+        </is>
+      </c>
       <c r="AE16" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.3500 (market_slug=aec-cs2-nvo-mouzn-2026-07-28).</t>
+          <t>Neutral Elo baseline; executable ask 0.5900 (market_slug=aec-cs2-ent-mta-2026-07-28).</t>
         </is>
       </c>
       <c r="AF16" s="31" t="inlineStr">
@@ -5547,32 +5575,32 @@
       </c>
       <c r="AP16" s="24" t="inlineStr">
         <is>
-          <t>MOUZ NXT</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="AQ16" s="24" t="inlineStr">
         <is>
-          <t>MOUZ NXT</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="AR16" s="24" t="inlineStr">
         <is>
-          <t>MOUZ NXT</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="AS16" s="24" t="inlineStr">
         <is>
-          <t>Noir Verse</t>
+          <t>Entropy</t>
         </is>
       </c>
       <c r="AT16" s="24" t="inlineStr">
         <is>
-          <t>Noir Verse</t>
+          <t>Entropy</t>
         </is>
       </c>
       <c r="AU16" s="24" t="inlineStr">
         <is>
-          <t>Noir Verse</t>
+          <t>Entropy</t>
         </is>
       </c>
       <c r="AV16" s="24" t="n"/>
@@ -5590,7 +5618,7 @@
       </c>
       <c r="BA16" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>40c2937bc668bb862cf7af94b4e50bd7f49459da4b5b52e8a268f7bbef6d0377</t>
         </is>
       </c>
       <c r="BB16" s="24" t="inlineStr">
@@ -5605,7 +5633,7 @@
       </c>
       <c r="BD16" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>40c2937bc668bb862cf7af94b4e50bd7f49459da4b5b52e8a268f7bbef6d0377</t>
         </is>
       </c>
       <c r="BE16" s="24" t="inlineStr">
@@ -5625,7 +5653,7 @@
       </c>
       <c r="BH16" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:40.889369Z</t>
+          <t>2026-07-28T05:05:26.235601Z</t>
         </is>
       </c>
       <c r="BI16" s="24" t="inlineStr">
@@ -5635,13 +5663,13 @@
       </c>
       <c r="BJ16" s="25" t="n"/>
       <c r="BK16" s="26" t="n">
-        <v>186</v>
+        <v>-144</v>
       </c>
       <c r="BL16" s="27" t="n">
-        <v>2.86</v>
+        <v>1.694444</v>
       </c>
       <c r="BM16" s="28" t="n">
-        <v>0.34965</v>
+        <v>0.590164</v>
       </c>
       <c r="BN16" s="28" t="n"/>
       <c r="BO16" s="28" t="n"/>
@@ -5675,22 +5703,22 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>8b7742d48b154a4c</t>
+          <t>d680f0c63c144b2a</t>
         </is>
       </c>
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T08:11:54.722189Z</t>
         </is>
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T11:00:00Z</t>
+          <t>2026-07-28T10:00:00Z</t>
         </is>
       </c>
       <c r="D17" s="24" t="inlineStr">
         <is>
-          <t>63359</t>
+          <t>64432</t>
         </is>
       </c>
       <c r="E17" s="24" t="inlineStr">
@@ -5700,12 +5728,12 @@
       </c>
       <c r="F17" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>MOUZ NXT</t>
         </is>
       </c>
       <c r="G17" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Noir Verse</t>
         </is>
       </c>
       <c r="H17" s="24" t="inlineStr">
@@ -5715,7 +5743,7 @@
       </c>
       <c r="I17" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J17" s="25" t="n"/>
@@ -5725,26 +5753,26 @@
         </is>
       </c>
       <c r="L17" s="26" t="n">
-        <v>-108</v>
+        <v>150</v>
       </c>
       <c r="M17" s="27" t="n">
-        <v>1.925926</v>
+        <v>2.5</v>
       </c>
       <c r="N17" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.4</v>
       </c>
       <c r="O17" s="28" t="n">
-        <v>0.589686</v>
+        <v>0.509533</v>
       </c>
       <c r="P17" s="28" t="n"/>
       <c r="Q17" s="28" t="n">
-        <v>0.070455</v>
+        <v>0.109533</v>
       </c>
       <c r="R17" s="26" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="S17" s="29" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="T17" s="24" t="inlineStr">
         <is>
@@ -5753,21 +5781,35 @@
       </c>
       <c r="U17" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V17" s="24" t="n"/>
-      <c r="W17" s="26" t="n"/>
-      <c r="X17" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V17" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X17" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y17" s="25" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="30" t="n"/>
-      <c r="AD17" s="24" t="n"/>
+      <c r="AC17" s="30" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AD17" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T14:18:45.452613Z</t>
+        </is>
+      </c>
       <c r="AE17" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5200 (market_slug=aec-cs2-btf-g2a-2026-07-28).</t>
+          <t>Neutral Elo baseline; executable ask 0.4000 (market_slug=aec-cs2-nvo-mouzn-2026-07-28).</t>
         </is>
       </c>
       <c r="AF17" s="31" t="inlineStr">
@@ -5777,7 +5819,7 @@
       </c>
       <c r="AG17" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH17" s="24" t="n"/>
@@ -5808,32 +5850,32 @@
       </c>
       <c r="AP17" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>MOUZ NXT</t>
         </is>
       </c>
       <c r="AQ17" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>MOUZ NXT</t>
         </is>
       </c>
       <c r="AR17" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>MOUZ NXT</t>
         </is>
       </c>
       <c r="AS17" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Noir Verse</t>
         </is>
       </c>
       <c r="AT17" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Noir Verse</t>
         </is>
       </c>
       <c r="AU17" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Noir Verse</t>
         </is>
       </c>
       <c r="AV17" s="24" t="n"/>
@@ -5851,7 +5893,7 @@
       </c>
       <c r="BA17" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>bc55e868a05b19a7a0abd9e0981ea1ca6d73030b07b9e89e745ea990df232cdb</t>
         </is>
       </c>
       <c r="BB17" s="24" t="inlineStr">
@@ -5866,7 +5908,7 @@
       </c>
       <c r="BD17" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>bc55e868a05b19a7a0abd9e0981ea1ca6d73030b07b9e89e745ea990df232cdb</t>
         </is>
       </c>
       <c r="BE17" s="24" t="inlineStr">
@@ -5886,7 +5928,7 @@
       </c>
       <c r="BH17" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:42.419976Z</t>
+          <t>2026-07-28T08:11:31.472875Z</t>
         </is>
       </c>
       <c r="BI17" s="24" t="inlineStr">
@@ -5896,13 +5938,13 @@
       </c>
       <c r="BJ17" s="25" t="n"/>
       <c r="BK17" s="26" t="n">
-        <v>-108</v>
+        <v>150</v>
       </c>
       <c r="BL17" s="27" t="n">
-        <v>1.925926</v>
+        <v>2.5</v>
       </c>
       <c r="BM17" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.4</v>
       </c>
       <c r="BN17" s="28" t="n"/>
       <c r="BO17" s="28" t="n"/>
@@ -5936,12 +5978,12 @@
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>f01f527cad484709</t>
+          <t>1230e8ccb3f14468</t>
         </is>
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T08:11:54.722189Z</t>
         </is>
       </c>
       <c r="C18" s="24" t="inlineStr">
@@ -5951,7 +5993,7 @@
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>64367</t>
+          <t>63359</t>
         </is>
       </c>
       <c r="E18" s="24" t="inlineStr">
@@ -5961,12 +6003,12 @@
       </c>
       <c r="F18" s="24" t="inlineStr">
         <is>
-          <t>Bebop</t>
+          <t>G2 Ares</t>
         </is>
       </c>
       <c r="G18" s="24" t="inlineStr">
         <is>
-          <t>Black Phoenix</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H18" s="24" t="inlineStr">
@@ -5986,26 +6028,26 @@
         </is>
       </c>
       <c r="L18" s="26" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="M18" s="27" t="n">
-        <v>2.17</v>
+        <v>2</v>
       </c>
       <c r="N18" s="28" t="n">
-        <v>0.460829</v>
+        <v>0.5</v>
       </c>
       <c r="O18" s="28" t="n">
-        <v>0.525641</v>
+        <v>0.589686</v>
       </c>
       <c r="P18" s="28" t="n"/>
       <c r="Q18" s="28" t="n">
-        <v>0.06481199999999999</v>
+        <v>0.089686</v>
       </c>
       <c r="R18" s="26" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="S18" s="29" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="T18" s="24" t="inlineStr">
         <is>
@@ -6014,21 +6056,35 @@
       </c>
       <c r="U18" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V18" s="24" t="n"/>
-      <c r="W18" s="26" t="n"/>
-      <c r="X18" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V18" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W18" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y18" s="25" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="30" t="n"/>
-      <c r="AD18" s="24" t="n"/>
+      <c r="AC18" s="30" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="AD18" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T14:18:46.743433Z</t>
+        </is>
+      </c>
       <c r="AE18" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.4600 (market_slug=aec-cs2-bpl-bbp-2026-07-28).</t>
+          <t>Neutral Elo baseline; executable ask 0.5000 (market_slug=aec-cs2-btf-g2a-2026-07-28).</t>
         </is>
       </c>
       <c r="AF18" s="31" t="inlineStr">
@@ -6038,7 +6094,7 @@
       </c>
       <c r="AG18" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH18" s="24" t="n"/>
@@ -6069,32 +6125,32 @@
       </c>
       <c r="AP18" s="24" t="inlineStr">
         <is>
-          <t>Bebop</t>
+          <t>G2 Ares</t>
         </is>
       </c>
       <c r="AQ18" s="24" t="inlineStr">
         <is>
-          <t>Bebop</t>
+          <t>G2 Ares</t>
         </is>
       </c>
       <c r="AR18" s="24" t="inlineStr">
         <is>
-          <t>Bebop</t>
+          <t>G2 Ares</t>
         </is>
       </c>
       <c r="AS18" s="24" t="inlineStr">
         <is>
-          <t>Black Phoenix</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AT18" s="24" t="inlineStr">
         <is>
-          <t>Black Phoenix</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AU18" s="24" t="inlineStr">
         <is>
-          <t>Black Phoenix</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AV18" s="24" t="n"/>
@@ -6112,7 +6168,7 @@
       </c>
       <c r="BA18" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>bc55e868a05b19a7a0abd9e0981ea1ca6d73030b07b9e89e745ea990df232cdb</t>
         </is>
       </c>
       <c r="BB18" s="24" t="inlineStr">
@@ -6127,7 +6183,7 @@
       </c>
       <c r="BD18" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>bc55e868a05b19a7a0abd9e0981ea1ca6d73030b07b9e89e745ea990df232cdb</t>
         </is>
       </c>
       <c r="BE18" s="24" t="inlineStr">
@@ -6147,7 +6203,7 @@
       </c>
       <c r="BH18" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:42.912018Z</t>
+          <t>2026-07-28T08:11:32.486834Z</t>
         </is>
       </c>
       <c r="BI18" s="24" t="inlineStr">
@@ -6157,13 +6213,13 @@
       </c>
       <c r="BJ18" s="25" t="n"/>
       <c r="BK18" s="26" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="BL18" s="27" t="n">
-        <v>2.17</v>
+        <v>2</v>
       </c>
       <c r="BM18" s="28" t="n">
-        <v>0.460829</v>
+        <v>0.5</v>
       </c>
       <c r="BN18" s="28" t="n"/>
       <c r="BO18" s="28" t="n"/>
@@ -6197,22 +6253,22 @@
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>a1ff007a7d104399</t>
+          <t>f939627a80c7422c</t>
         </is>
       </c>
       <c r="B19" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T08:11:54.722189Z</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T14:00:00Z</t>
+          <t>2026-07-28T11:00:00Z</t>
         </is>
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>63360</t>
+          <t>64367</t>
         </is>
       </c>
       <c r="E19" s="24" t="inlineStr">
@@ -6222,12 +6278,12 @@
       </c>
       <c r="F19" s="24" t="inlineStr">
         <is>
-          <t>Just Players</t>
+          <t>Bebop</t>
         </is>
       </c>
       <c r="G19" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="H19" s="24" t="inlineStr">
@@ -6247,49 +6303,63 @@
         </is>
       </c>
       <c r="L19" s="26" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="M19" s="27" t="n">
-        <v>2.08</v>
+        <v>2.13</v>
       </c>
       <c r="N19" s="28" t="n">
-        <v>0.480769</v>
+        <v>0.469484</v>
       </c>
       <c r="O19" s="28" t="n">
-        <v>0.53791</v>
+        <v>0.525641</v>
       </c>
       <c r="P19" s="28" t="n"/>
       <c r="Q19" s="28" t="n">
-        <v>0.057141</v>
+        <v>0.056157</v>
       </c>
       <c r="R19" s="26" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S19" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T19" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v4</t>
+        </is>
+      </c>
+      <c r="U19" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V19" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W19" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="T19" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v4</t>
-        </is>
-      </c>
-      <c r="U19" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V19" s="24" t="n"/>
-      <c r="W19" s="26" t="n"/>
-      <c r="X19" s="26" t="n"/>
+      <c r="X19" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y19" s="25" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="30" t="n"/>
-      <c r="AD19" s="24" t="n"/>
+      <c r="AC19" s="30" t="n">
+        <v>0.8475</v>
+      </c>
+      <c r="AD19" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T14:18:47.865907Z</t>
+        </is>
+      </c>
       <c r="AE19" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.4800 (market_slug=aec-cs2-btf-jpu-2026-07-28).</t>
+          <t>Neutral Elo baseline; executable ask 0.4700 (market_slug=aec-cs2-bpl-bbp-2026-07-28).</t>
         </is>
       </c>
       <c r="AF19" s="31" t="inlineStr">
@@ -6330,32 +6400,32 @@
       </c>
       <c r="AP19" s="24" t="inlineStr">
         <is>
-          <t>Just Players</t>
+          <t>Bebop</t>
         </is>
       </c>
       <c r="AQ19" s="24" t="inlineStr">
         <is>
-          <t>Just Players</t>
+          <t>Bebop</t>
         </is>
       </c>
       <c r="AR19" s="24" t="inlineStr">
         <is>
-          <t>Just Players</t>
+          <t>Bebop</t>
         </is>
       </c>
       <c r="AS19" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="AT19" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="AU19" s="24" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Black Phoenix</t>
         </is>
       </c>
       <c r="AV19" s="24" t="n"/>
@@ -6373,7 +6443,7 @@
       </c>
       <c r="BA19" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>bc55e868a05b19a7a0abd9e0981ea1ca6d73030b07b9e89e745ea990df232cdb</t>
         </is>
       </c>
       <c r="BB19" s="24" t="inlineStr">
@@ -6388,7 +6458,7 @@
       </c>
       <c r="BD19" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>bc55e868a05b19a7a0abd9e0981ea1ca6d73030b07b9e89e745ea990df232cdb</t>
         </is>
       </c>
       <c r="BE19" s="24" t="inlineStr">
@@ -6408,7 +6478,7 @@
       </c>
       <c r="BH19" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:45.363088Z</t>
+          <t>2026-07-28T08:11:33.028196Z</t>
         </is>
       </c>
       <c r="BI19" s="24" t="inlineStr">
@@ -6418,13 +6488,13 @@
       </c>
       <c r="BJ19" s="25" t="n"/>
       <c r="BK19" s="26" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="BL19" s="27" t="n">
-        <v>2.08</v>
+        <v>2.13</v>
       </c>
       <c r="BM19" s="28" t="n">
-        <v>0.480769</v>
+        <v>0.469484</v>
       </c>
       <c r="BN19" s="28" t="n"/>
       <c r="BO19" s="28" t="n"/>
@@ -6458,22 +6528,22 @@
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>147b001ceaa24335</t>
+          <t>0961e2f1cea44460</t>
         </is>
       </c>
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T11:17:59.302295Z</t>
         </is>
       </c>
       <c r="C20" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T17:00:00Z</t>
+          <t>2026-07-28T14:00:00Z</t>
         </is>
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>63362</t>
+          <t>63360</t>
         </is>
       </c>
       <c r="E20" s="24" t="inlineStr">
@@ -6483,12 +6553,12 @@
       </c>
       <c r="F20" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Just Players</t>
         </is>
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H20" s="24" t="inlineStr">
@@ -6508,23 +6578,23 @@
         </is>
       </c>
       <c r="L20" s="26" t="n">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="M20" s="27" t="n">
-        <v>2.27</v>
+        <v>2.13</v>
       </c>
       <c r="N20" s="28" t="n">
-        <v>0.440529</v>
+        <v>0.469484</v>
       </c>
       <c r="O20" s="28" t="n">
-        <v>0.548241</v>
+        <v>0.53772</v>
       </c>
       <c r="P20" s="28" t="n"/>
       <c r="Q20" s="28" t="n">
-        <v>0.107712</v>
+        <v>0.068236</v>
       </c>
       <c r="R20" s="26" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="S20" s="29" t="n">
         <v>1</v>
@@ -6550,7 +6620,7 @@
       <c r="AD20" s="24" t="n"/>
       <c r="AE20" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.4400 (market_slug=aec-cs2-sparta-g2a-2026-07-28).</t>
+          <t>Neutral Elo baseline; executable ask 0.4700 (market_slug=aec-cs2-btf-jpu-2026-07-28).</t>
         </is>
       </c>
       <c r="AF20" s="31" t="inlineStr">
@@ -6591,32 +6661,32 @@
       </c>
       <c r="AP20" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Just Players</t>
         </is>
       </c>
       <c r="AQ20" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Just Players</t>
         </is>
       </c>
       <c r="AR20" s="24" t="inlineStr">
         <is>
-          <t>G2 Ares</t>
+          <t>Just Players</t>
         </is>
       </c>
       <c r="AS20" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AT20" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AU20" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="AV20" s="24" t="n"/>
@@ -6634,7 +6704,7 @@
       </c>
       <c r="BA20" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>2b10a508f0b7c33f18d6ceeb867088d36516a5ff42abbccd848c68e2c7ca105c</t>
         </is>
       </c>
       <c r="BB20" s="24" t="inlineStr">
@@ -6649,7 +6719,7 @@
       </c>
       <c r="BD20" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>2b10a508f0b7c33f18d6ceeb867088d36516a5ff42abbccd848c68e2c7ca105c</t>
         </is>
       </c>
       <c r="BE20" s="24" t="inlineStr">
@@ -6669,7 +6739,7 @@
       </c>
       <c r="BH20" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:47.940507Z</t>
+          <t>2026-07-28T11:17:40.063714Z</t>
         </is>
       </c>
       <c r="BI20" s="24" t="inlineStr">
@@ -6679,13 +6749,13 @@
       </c>
       <c r="BJ20" s="25" t="n"/>
       <c r="BK20" s="26" t="n">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="BL20" s="27" t="n">
-        <v>2.27</v>
+        <v>2.13</v>
       </c>
       <c r="BM20" s="28" t="n">
-        <v>0.440529</v>
+        <v>0.469484</v>
       </c>
       <c r="BN20" s="28" t="n"/>
       <c r="BO20" s="28" t="n"/>
@@ -6719,22 +6789,22 @@
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>2b723c7fba9643ee</t>
+          <t>3ade7d7fea21469e</t>
         </is>
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T02:00:01.501477Z</t>
+          <t>2026-07-28T14:24:09.023643Z</t>
         </is>
       </c>
       <c r="C21" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T17:00:00Z</t>
+          <t>2026-07-28T15:00:00Z</t>
         </is>
       </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
-          <t>63363</t>
+          <t>61517</t>
         </is>
       </c>
       <c r="E21" s="24" t="inlineStr">
@@ -6744,12 +6814,12 @@
       </c>
       <c r="F21" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>BakS eSports</t>
         </is>
       </c>
       <c r="G21" s="24" t="inlineStr">
         <is>
-          <t>CYBERSHOKE Prospects</t>
+          <t>TDK</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">
@@ -6759,7 +6829,7 @@
       </c>
       <c r="I21" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J21" s="25" t="n"/>
@@ -6769,26 +6839,26 @@
         </is>
       </c>
       <c r="L21" s="26" t="n">
-        <v>113</v>
+        <v>-194</v>
       </c>
       <c r="M21" s="27" t="n">
-        <v>2.13</v>
+        <v>1.515464</v>
       </c>
       <c r="N21" s="28" t="n">
-        <v>0.469484</v>
+        <v>0.659864</v>
       </c>
       <c r="O21" s="28" t="n">
-        <v>0.553566</v>
+        <v>0.907919</v>
       </c>
       <c r="P21" s="28" t="n"/>
       <c r="Q21" s="28" t="n">
-        <v>0.084082</v>
+        <v>0.248055</v>
       </c>
       <c r="R21" s="26" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="S21" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T21" s="24" t="inlineStr">
         <is>
@@ -6811,7 +6881,7 @@
       <c r="AD21" s="24" t="n"/>
       <c r="AE21" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.4700 (market_slug=aec-cs2-cshp-lav-2026-07-28).</t>
+          <t>Neutral Elo baseline; executable ask 0.6600 (market_slug=aec-cs2-tdk-baks-2026-07-28).</t>
         </is>
       </c>
       <c r="AF21" s="31" t="inlineStr">
@@ -6852,32 +6922,32 @@
       </c>
       <c r="AP21" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>BakS eSports</t>
         </is>
       </c>
       <c r="AQ21" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>BakS eSports</t>
         </is>
       </c>
       <c r="AR21" s="24" t="inlineStr">
         <is>
-          <t>Lavked</t>
+          <t>BakS eSports</t>
         </is>
       </c>
       <c r="AS21" s="24" t="inlineStr">
         <is>
-          <t>CYBERSHOKE Prospects</t>
+          <t>TDK</t>
         </is>
       </c>
       <c r="AT21" s="24" t="inlineStr">
         <is>
-          <t>CYBERSHOKE Prospects</t>
+          <t>TDK</t>
         </is>
       </c>
       <c r="AU21" s="24" t="inlineStr">
         <is>
-          <t>CYBERSHOKE Prospects</t>
+          <t>TDK</t>
         </is>
       </c>
       <c r="AV21" s="24" t="n"/>
@@ -6895,7 +6965,7 @@
       </c>
       <c r="BA21" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>b7be26981f98c7c049773609859384b830ed2600e5d283ac2efb1545695d5e3e</t>
         </is>
       </c>
       <c r="BB21" s="24" t="inlineStr">
@@ -6910,7 +6980,7 @@
       </c>
       <c r="BD21" s="24" t="inlineStr">
         <is>
-          <t>da5537802607ba1fbdae985f92f1b67c327aaa91913ae14bcd767a484004f207</t>
+          <t>b7be26981f98c7c049773609859384b830ed2600e5d283ac2efb1545695d5e3e</t>
         </is>
       </c>
       <c r="BE21" s="24" t="inlineStr">
@@ -6930,7 +7000,7 @@
       </c>
       <c r="BH21" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T01:59:49.411771Z</t>
+          <t>2026-07-28T14:23:49.113149Z</t>
         </is>
       </c>
       <c r="BI21" s="24" t="inlineStr">
@@ -6940,13 +7010,13 @@
       </c>
       <c r="BJ21" s="25" t="n"/>
       <c r="BK21" s="26" t="n">
-        <v>113</v>
+        <v>-194</v>
       </c>
       <c r="BL21" s="27" t="n">
-        <v>2.13</v>
+        <v>1.515464</v>
       </c>
       <c r="BM21" s="28" t="n">
-        <v>0.469484</v>
+        <v>0.659864</v>
       </c>
       <c r="BN21" s="28" t="n"/>
       <c r="BO21" s="28" t="n"/>
@@ -6977,267 +7047,6 @@
       <c r="CN21" s="24" t="n"/>
       <c r="CO21" s="24" t="n"/>
     </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
-        <is>
-          <t>98542e97ce3841ee</t>
-        </is>
-      </c>
-      <c r="B22" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-28T02:08:42.519814Z</t>
-        </is>
-      </c>
-      <c r="C22" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-28T08:00:00Z</t>
-        </is>
-      </c>
-      <c r="D22" s="24" t="inlineStr">
-        <is>
-          <t>63706</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr">
-        <is>
-          <t>Mai Tai</t>
-        </is>
-      </c>
-      <c r="G22" s="24" t="inlineStr">
-        <is>
-          <t>Entropy</t>
-        </is>
-      </c>
-      <c r="H22" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I22" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J22" s="25" t="n"/>
-      <c r="K22" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L22" s="26" t="n">
-        <v>-138</v>
-      </c>
-      <c r="M22" s="27" t="n">
-        <v>1.724638</v>
-      </c>
-      <c r="N22" s="28" t="n">
-        <v>0.579832</v>
-      </c>
-      <c r="O22" s="28" t="n">
-        <v>0.609287</v>
-      </c>
-      <c r="P22" s="28" t="n"/>
-      <c r="Q22" s="28" t="n">
-        <v>0.029455</v>
-      </c>
-      <c r="R22" s="26" t="n">
-        <v>35</v>
-      </c>
-      <c r="S22" s="29" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="T22" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v4</t>
-        </is>
-      </c>
-      <c r="U22" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V22" s="24" t="n"/>
-      <c r="W22" s="26" t="n"/>
-      <c r="X22" s="26" t="n"/>
-      <c r="Y22" s="25" t="n"/>
-      <c r="Z22" s="26" t="n"/>
-      <c r="AA22" s="28" t="n"/>
-      <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="30" t="n"/>
-      <c r="AD22" s="24" t="n"/>
-      <c r="AE22" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-ent-mta-2026-07-28).</t>
-        </is>
-      </c>
-      <c r="AF22" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG22" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH22" s="24" t="n"/>
-      <c r="AI22" s="31" t="n"/>
-      <c r="AJ22" s="31" t="n"/>
-      <c r="AK22" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL22" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM22" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN22" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO22" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP22" s="24" t="inlineStr">
-        <is>
-          <t>Mai Tai</t>
-        </is>
-      </c>
-      <c r="AQ22" s="24" t="inlineStr">
-        <is>
-          <t>Mai Tai</t>
-        </is>
-      </c>
-      <c r="AR22" s="24" t="inlineStr">
-        <is>
-          <t>Mai Tai</t>
-        </is>
-      </c>
-      <c r="AS22" s="24" t="inlineStr">
-        <is>
-          <t>Entropy</t>
-        </is>
-      </c>
-      <c r="AT22" s="24" t="inlineStr">
-        <is>
-          <t>Entropy</t>
-        </is>
-      </c>
-      <c r="AU22" s="24" t="inlineStr">
-        <is>
-          <t>Entropy</t>
-        </is>
-      </c>
-      <c r="AV22" s="24" t="n"/>
-      <c r="AW22" s="24" t="n"/>
-      <c r="AX22" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY22" s="24" t="n"/>
-      <c r="AZ22" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA22" s="24" t="inlineStr">
-        <is>
-          <t>083967481304d1dc27bfb10e14bb394ac08ceeda4b7f4e87080bc0131a2aed37</t>
-        </is>
-      </c>
-      <c r="BB22" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC22" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v4</t>
-        </is>
-      </c>
-      <c r="BD22" s="24" t="inlineStr">
-        <is>
-          <t>083967481304d1dc27bfb10e14bb394ac08ceeda4b7f4e87080bc0131a2aed37</t>
-        </is>
-      </c>
-      <c r="BE22" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF22" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG22" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v4</t>
-        </is>
-      </c>
-      <c r="BH22" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-28T02:08:19.728443Z</t>
-        </is>
-      </c>
-      <c r="BI22" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ22" s="25" t="n"/>
-      <c r="BK22" s="26" t="n">
-        <v>-138</v>
-      </c>
-      <c r="BL22" s="27" t="n">
-        <v>1.724638</v>
-      </c>
-      <c r="BM22" s="28" t="n">
-        <v>0.579832</v>
-      </c>
-      <c r="BN22" s="28" t="n"/>
-      <c r="BO22" s="28" t="n"/>
-      <c r="BP22" s="25" t="n"/>
-      <c r="BQ22" s="27" t="n"/>
-      <c r="BR22" s="28" t="n"/>
-      <c r="BS22" s="28" t="n"/>
-      <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="25" t="n"/>
-      <c r="BV22" s="29" t="n"/>
-      <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="30" t="n"/>
-      <c r="BY22" s="27" t="n"/>
-      <c r="BZ22" s="24" t="n"/>
-      <c r="CA22" s="31" t="n"/>
-      <c r="CB22" s="24" t="n"/>
-      <c r="CC22" s="24" t="n"/>
-      <c r="CD22" s="24" t="n"/>
-      <c r="CE22" s="24" t="n"/>
-      <c r="CF22" s="24" t="n"/>
-      <c r="CG22" s="24" t="n"/>
-      <c r="CH22" s="24" t="n"/>
-      <c r="CI22" s="24" t="n"/>
-      <c r="CJ22" s="24" t="n"/>
-      <c r="CK22" s="24" t="n"/>
-      <c r="CL22" s="24" t="n"/>
-      <c r="CM22" s="24" t="n"/>
-      <c r="CN22" s="24" t="n"/>
-      <c r="CO22" s="24" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Sync ledger/eligibility work: model_ledger module, research/gated-research reorg, live data through 8/2
Adds src/model_prediction/model_ledger.py + migration script, docs/HISTORY.md
and MASTER.md, expanded test coverage (test_model_ledger.py, test_research_io.py,
plus substantial additions across existing test files). Bundles the accumulated
operational data (ledger xlsx files, ESPN/Polymarket snapshots, WNBA availability
captures) from running the pipeline through 2026-08-02.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,9 +300,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO15" headerRowCount="1">
-  <autoFilter ref="A1:CO15"/>
-  <tableColumns count="93">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CP14" headerRowCount="1">
+  <autoFilter ref="A1:CP14"/>
+  <tableColumns count="94">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
     <tableColumn id="3" name="event_start_utc"/>
@@ -396,6 +396,7 @@
     <tableColumn id="91" name="back_to_back_gap"/>
     <tableColumn id="92" name="games_last_7_gap"/>
     <tableColumn id="93" name="schedule_missingness"/>
+    <tableColumn id="94" name="trade_candidate"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -752,19 +753,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$15)</f>
+        <f>COUNTA('Picks'!$A$2:$A$14)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$15,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")+COUNTIFS('Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -792,19 +793,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$15,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"win")/(COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"win")+COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$15)/SUM('Picks'!$BX$2:$BX$15),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
         <v/>
       </c>
     </row>
@@ -832,19 +833,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$15)</f>
+        <f>SUM('Picks'!$BY$2:$BY$14)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$15,"&lt;&gt;",'Picks'!$AB$2:$AB$15),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$15,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$15,'Picks'!$AM$2:$AM$15,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -899,15 +900,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -915,11 +916,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$15,'Picks'!$H$2:$H$15,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$15,'Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -930,15 +931,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -946,11 +947,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$15,'Picks'!$H$2:$H$15,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$15,'Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -961,15 +962,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -977,11 +978,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$15,'Picks'!$H$2:$H$15,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$15,'Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1010,7 +1011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CO15"/>
+  <dimension ref="A1:CP14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1106,6 +1107,7 @@
     <col width="18" customWidth="1" min="91" max="91"/>
     <col width="18" customWidth="1" min="92" max="92"/>
     <col width="22" customWidth="1" min="93" max="93"/>
+    <col width="17" customWidth="1" min="94" max="94"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1572,6 +1574,11 @@
       <c r="CO1" s="23" t="inlineStr">
         <is>
           <t>schedule_missingness</t>
+        </is>
+      </c>
+      <c r="CP1" s="23" t="inlineStr">
+        <is>
+          <t>trade_candidate</t>
         </is>
       </c>
     </row>
@@ -1859,6 +1866,7 @@
       <c r="CM2" s="24" t="n"/>
       <c r="CN2" s="24" t="n"/>
       <c r="CO2" s="24" t="n"/>
+      <c r="CP2" s="24" t="n"/>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
@@ -2144,6 +2152,7 @@
       <c r="CM3" s="24" t="n"/>
       <c r="CN3" s="24" t="n"/>
       <c r="CO3" s="24" t="n"/>
+      <c r="CP3" s="24" t="n"/>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -2429,6 +2438,7 @@
       <c r="CM4" s="24" t="n"/>
       <c r="CN4" s="24" t="n"/>
       <c r="CO4" s="24" t="n"/>
+      <c r="CP4" s="24" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
@@ -2714,6 +2724,7 @@
       <c r="CM5" s="24" t="n"/>
       <c r="CN5" s="24" t="n"/>
       <c r="CO5" s="24" t="n"/>
+      <c r="CP5" s="24" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -2999,6 +3010,7 @@
       <c r="CM6" s="24" t="n"/>
       <c r="CN6" s="24" t="n"/>
       <c r="CO6" s="24" t="n"/>
+      <c r="CP6" s="24" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
@@ -3284,6 +3296,7 @@
       <c r="CM7" s="24" t="n"/>
       <c r="CN7" s="24" t="n"/>
       <c r="CO7" s="24" t="n"/>
+      <c r="CP7" s="24" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -3569,6 +3582,7 @@
       <c r="CM8" s="24" t="n"/>
       <c r="CN8" s="24" t="n"/>
       <c r="CO8" s="24" t="n"/>
+      <c r="CP8" s="24" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
@@ -3854,6 +3868,7 @@
       <c r="CM9" s="24" t="n"/>
       <c r="CN9" s="24" t="n"/>
       <c r="CO9" s="24" t="n"/>
+      <c r="CP9" s="24" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -4139,6 +4154,7 @@
       <c r="CM10" s="24" t="n"/>
       <c r="CN10" s="24" t="n"/>
       <c r="CO10" s="24" t="n"/>
+      <c r="CP10" s="24" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
@@ -4424,6 +4440,7 @@
       <c r="CM11" s="24" t="n"/>
       <c r="CN11" s="24" t="n"/>
       <c r="CO11" s="24" t="n"/>
+      <c r="CP11" s="24" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -4685,16 +4702,17 @@
       <c r="CM12" s="24" t="n"/>
       <c r="CN12" s="24" t="n"/>
       <c r="CO12" s="24" t="n"/>
+      <c r="CP12" s="24" t="n"/>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>1266e5481bb746cc</t>
+          <t>1890098872ae4443</t>
         </is>
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T10:00:04.561525Z</t>
+          <t>2026-08-02T12:30:33.225632Z</t>
         </is>
       </c>
       <c r="C13" s="24" t="inlineStr">
@@ -4748,11 +4766,11 @@
         <v>0.530516</v>
       </c>
       <c r="O13" s="28" t="n">
-        <v>0.676069</v>
+        <v>0.67594</v>
       </c>
       <c r="P13" s="28" t="n"/>
       <c r="Q13" s="28" t="n">
-        <v>0.145553</v>
+        <v>0.145424</v>
       </c>
       <c r="R13" s="26" t="n">
         <v>93</v>
@@ -4865,7 +4883,7 @@
       </c>
       <c r="BA13" s="24" t="inlineStr">
         <is>
-          <t>06138ffc8334cb69044b84c6e2b37aa9a4e0b6bd4f08ef7c62950d9e210f4364</t>
+          <t>bd7b44b2e86615e932309b2497f806ee2b5567367d785a2c9653f7a6fe2215fb</t>
         </is>
       </c>
       <c r="BB13" s="24" t="inlineStr">
@@ -4880,7 +4898,7 @@
       </c>
       <c r="BD13" s="24" t="inlineStr">
         <is>
-          <t>06138ffc8334cb69044b84c6e2b37aa9a4e0b6bd4f08ef7c62950d9e210f4364</t>
+          <t>bd7b44b2e86615e932309b2497f806ee2b5567367d785a2c9653f7a6fe2215fb</t>
         </is>
       </c>
       <c r="BE13" s="24" t="inlineStr">
@@ -4900,7 +4918,7 @@
       </c>
       <c r="BH13" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T09:59:46.682984Z</t>
+          <t>2026-08-02T12:30:14.025736Z</t>
         </is>
       </c>
       <c r="BI13" s="24" t="inlineStr">
@@ -4946,16 +4964,17 @@
       <c r="CM13" s="24" t="n"/>
       <c r="CN13" s="24" t="n"/>
       <c r="CO13" s="24" t="n"/>
+      <c r="CP13" s="24" t="n"/>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>049e2112fd6048d2</t>
+          <t>2dc39e41acdf4581</t>
         </is>
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T10:00:04.561525Z</t>
+          <t>2026-08-02T13:07:50.282319Z</t>
         </is>
       </c>
       <c r="C14" s="24" t="inlineStr">
@@ -5000,23 +5019,23 @@
         </is>
       </c>
       <c r="L14" s="26" t="n">
-        <v>-156</v>
+        <v>-170</v>
       </c>
       <c r="M14" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.588235</v>
       </c>
       <c r="N14" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.62963</v>
       </c>
       <c r="O14" s="28" t="n">
-        <v>0.66636</v>
+        <v>0.6659040000000001</v>
       </c>
       <c r="P14" s="28" t="n"/>
       <c r="Q14" s="28" t="n">
-        <v>0.056985</v>
+        <v>0.036274</v>
       </c>
       <c r="R14" s="26" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="S14" s="29" t="n">
         <v>1.75</v>
@@ -5042,7 +5061,7 @@
       <c r="AD14" s="24" t="n"/>
       <c r="AE14" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6100 (market_slug=aec-cs2-mta-enjoy-2026-08-02).</t>
+          <t>Neutral Elo baseline; executable ask 0.6300 (market_slug=aec-cs2-mta-enjoy-2026-08-02).</t>
         </is>
       </c>
       <c r="AF14" s="31" t="inlineStr">
@@ -5126,7 +5145,7 @@
       </c>
       <c r="BA14" s="24" t="inlineStr">
         <is>
-          <t>06138ffc8334cb69044b84c6e2b37aa9a4e0b6bd4f08ef7c62950d9e210f4364</t>
+          <t>90a833898e793d48aa6ce23d298a692fd7b914cfa51b8101005c627e8a886f30</t>
         </is>
       </c>
       <c r="BB14" s="24" t="inlineStr">
@@ -5141,7 +5160,7 @@
       </c>
       <c r="BD14" s="24" t="inlineStr">
         <is>
-          <t>06138ffc8334cb69044b84c6e2b37aa9a4e0b6bd4f08ef7c62950d9e210f4364</t>
+          <t>90a833898e793d48aa6ce23d298a692fd7b914cfa51b8101005c627e8a886f30</t>
         </is>
       </c>
       <c r="BE14" s="24" t="inlineStr">
@@ -5161,7 +5180,7 @@
       </c>
       <c r="BH14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T09:59:51.297257Z</t>
+          <t>2026-08-02T13:07:36.093507Z</t>
         </is>
       </c>
       <c r="BI14" s="24" t="inlineStr">
@@ -5171,13 +5190,13 @@
       </c>
       <c r="BJ14" s="25" t="n"/>
       <c r="BK14" s="26" t="n">
-        <v>-156</v>
+        <v>-170</v>
       </c>
       <c r="BL14" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.588235</v>
       </c>
       <c r="BM14" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.62963</v>
       </c>
       <c r="BN14" s="28" t="n"/>
       <c r="BO14" s="28" t="n"/>
@@ -5207,267 +5226,7 @@
       <c r="CM14" s="24" t="n"/>
       <c r="CN14" s="24" t="n"/>
       <c r="CO14" s="24" t="n"/>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>043ff069ee9a43ae</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T10:00:04.561525Z</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T10:30:00Z</t>
-        </is>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>67514</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F15" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="G15" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="H15" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I15" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J15" s="25" t="n"/>
-      <c r="K15" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L15" s="26" t="n">
-        <v>-122</v>
-      </c>
-      <c r="M15" s="27" t="n">
-        <v>1.819672</v>
-      </c>
-      <c r="N15" s="28" t="n">
-        <v>0.54955</v>
-      </c>
-      <c r="O15" s="28" t="n">
-        <v>0.640228</v>
-      </c>
-      <c r="P15" s="28" t="n"/>
-      <c r="Q15" s="28" t="n">
-        <v>0.09067799999999999</v>
-      </c>
-      <c r="R15" s="26" t="n">
-        <v>65</v>
-      </c>
-      <c r="S15" s="29" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="T15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U15" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V15" s="24" t="n"/>
-      <c r="W15" s="26" t="n"/>
-      <c r="X15" s="26" t="n"/>
-      <c r="Y15" s="25" t="n"/>
-      <c r="Z15" s="26" t="n"/>
-      <c r="AA15" s="28" t="n"/>
-      <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n"/>
-      <c r="AD15" s="24" t="n"/>
-      <c r="AE15" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5500 (market_slug=aec-cs2-era-psna-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF15" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG15" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH15" s="24" t="n"/>
-      <c r="AI15" s="31" t="n"/>
-      <c r="AJ15" s="31" t="n"/>
-      <c r="AK15" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL15" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM15" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN15" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO15" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP15" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="AQ15" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="AR15" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="AS15" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="AT15" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="AU15" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="AV15" s="24" t="n"/>
-      <c r="AW15" s="24" t="n"/>
-      <c r="AX15" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY15" s="24" t="n"/>
-      <c r="AZ15" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA15" s="24" t="inlineStr">
-        <is>
-          <t>06138ffc8334cb69044b84c6e2b37aa9a4e0b6bd4f08ef7c62950d9e210f4364</t>
-        </is>
-      </c>
-      <c r="BB15" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD15" s="24" t="inlineStr">
-        <is>
-          <t>06138ffc8334cb69044b84c6e2b37aa9a4e0b6bd4f08ef7c62950d9e210f4364</t>
-        </is>
-      </c>
-      <c r="BE15" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF15" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T09:59:57.251438Z</t>
-        </is>
-      </c>
-      <c r="BI15" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ15" s="25" t="n"/>
-      <c r="BK15" s="26" t="n">
-        <v>-122</v>
-      </c>
-      <c r="BL15" s="27" t="n">
-        <v>1.819672</v>
-      </c>
-      <c r="BM15" s="28" t="n">
-        <v>0.54955</v>
-      </c>
-      <c r="BN15" s="28" t="n"/>
-      <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
-      <c r="BR15" s="28" t="n"/>
-      <c r="BS15" s="28" t="n"/>
-      <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="25" t="n"/>
-      <c r="BV15" s="29" t="n"/>
-      <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="30" t="n"/>
-      <c r="BY15" s="27" t="n"/>
-      <c r="BZ15" s="24" t="n"/>
-      <c r="CA15" s="31" t="n"/>
-      <c r="CB15" s="24" t="n"/>
-      <c r="CC15" s="24" t="n"/>
-      <c r="CD15" s="24" t="n"/>
-      <c r="CE15" s="24" t="n"/>
-      <c r="CF15" s="24" t="n"/>
-      <c r="CG15" s="24" t="n"/>
-      <c r="CH15" s="24" t="n"/>
-      <c r="CI15" s="24" t="n"/>
-      <c r="CJ15" s="24" t="n"/>
-      <c r="CK15" s="24" t="n"/>
-      <c r="CL15" s="24" t="n"/>
-      <c r="CM15" s="24" t="n"/>
-      <c r="CN15" s="24" t="n"/>
-      <c r="CO15" s="24" t="n"/>
+      <c r="CP14" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix soccer moneyline draw grading and model-ledger dedupe key; sync daily pipeline data
grade_pick() was treating a soccer draw as a push instead of a loss --
Polymarket's soccer win market is three independent Yes/No contracts, not
a single 2-outcome market with a tie, so a drawn "home"/"away" pick is a
full stake loss (KBO/NPB genuinely are 2-outcome ties and keep pushing).

ModelLedger's dedupe key omitted observed_at_utc, so a re-forecast of a
still-open pick (same event/market/line/model_version, new probability
and price) was silently dropped as a duplicate of the stale prior row.

Also includes accumulated daily-pipeline output since the last push:
esports/KBO/NPB ratings refresh with new rollback-safety .previous.json
snapshots, MLB availability captures, WNBA snapshots, ledger/odds data,
and README updates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CP14" headerRowCount="1">
-  <autoFilter ref="A1:CP14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CP16" headerRowCount="1">
+  <autoFilter ref="A1:CP16"/>
   <tableColumns count="94">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -753,19 +753,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$14)</f>
+        <f>COUNTA('Picks'!$A$2:$A$16)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$16,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -793,19 +793,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$16,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")/(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$16)/SUM('Picks'!$BX$2:$BX$16),0)</f>
         <v/>
       </c>
     </row>
@@ -833,19 +833,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$14)</f>
+        <f>SUM('Picks'!$BY$2:$BY$16)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$16,"&lt;&gt;",'Picks'!$AB$2:$AB$16),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$16,'Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -900,15 +900,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -916,11 +916,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -931,15 +931,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -947,11 +947,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -962,15 +962,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -978,11 +978,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CP14"/>
+  <dimension ref="A1:CP16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4523,18 +4523,28 @@
       </c>
       <c r="U12" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V12" s="24" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V12" s="24" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
       <c r="W12" s="26" t="n"/>
       <c r="X12" s="26" t="n"/>
       <c r="Y12" s="25" t="n"/>
       <c r="Z12" s="26" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="30" t="n"/>
-      <c r="AD12" s="24" t="n"/>
+      <c r="AC12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T15:53:33.702018Z</t>
+        </is>
+      </c>
       <c r="AE12" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.5100 (market_slug=aec-cs2-ttbs-sng-2026-08-02).</t>
@@ -4683,7 +4693,11 @@
       <c r="BT12" s="28" t="n"/>
       <c r="BU12" s="25" t="n"/>
       <c r="BV12" s="29" t="n"/>
-      <c r="BW12" s="24" t="n"/>
+      <c r="BW12" s="24" t="inlineStr">
+        <is>
+          <t>esports market settled to a non-binary price (forfeit/postponement per market rules)</t>
+        </is>
+      </c>
       <c r="BX12" s="30" t="n"/>
       <c r="BY12" s="27" t="n"/>
       <c r="BZ12" s="24" t="n"/>
@@ -4969,12 +4983,12 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>2dc39e41acdf4581</t>
+          <t>7c8a11062be44bbf</t>
         </is>
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T13:07:50.282319Z</t>
+          <t>2026-08-02T15:51:41.323824Z</t>
         </is>
       </c>
       <c r="C14" s="24" t="inlineStr">
@@ -4984,7 +4998,7 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>69263</t>
+          <t>69680</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
@@ -4994,12 +5008,12 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>ENJOY</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
         <is>
-          <t>Mai Tai</t>
+          <t>Fortress</t>
         </is>
       </c>
       <c r="H14" s="24" t="inlineStr">
@@ -5019,23 +5033,23 @@
         </is>
       </c>
       <c r="L14" s="26" t="n">
-        <v>-170</v>
+        <v>-156</v>
       </c>
       <c r="M14" s="27" t="n">
-        <v>1.588235</v>
+        <v>1.641026</v>
       </c>
       <c r="N14" s="28" t="n">
-        <v>0.62963</v>
+        <v>0.609375</v>
       </c>
       <c r="O14" s="28" t="n">
-        <v>0.6659040000000001</v>
+        <v>0.653037</v>
       </c>
       <c r="P14" s="28" t="n"/>
       <c r="Q14" s="28" t="n">
-        <v>0.036274</v>
+        <v>0.043662</v>
       </c>
       <c r="R14" s="26" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S14" s="29" t="n">
         <v>1.75</v>
@@ -5061,7 +5075,7 @@
       <c r="AD14" s="24" t="n"/>
       <c r="AE14" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6300 (market_slug=aec-cs2-mta-enjoy-2026-08-02).</t>
+          <t>Neutral Elo baseline; executable ask 0.6100 (market_slug=aec-cs2-for-lk-2026-08-02).</t>
         </is>
       </c>
       <c r="AF14" s="31" t="inlineStr">
@@ -5102,32 +5116,32 @@
       </c>
       <c r="AP14" s="24" t="inlineStr">
         <is>
-          <t>ENJOY</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="AQ14" s="24" t="inlineStr">
         <is>
-          <t>ENJOY</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="AR14" s="24" t="inlineStr">
         <is>
-          <t>ENJOY</t>
+          <t>los kogutos</t>
         </is>
       </c>
       <c r="AS14" s="24" t="inlineStr">
         <is>
-          <t>Mai Tai</t>
+          <t>Fortress</t>
         </is>
       </c>
       <c r="AT14" s="24" t="inlineStr">
         <is>
-          <t>Mai Tai</t>
+          <t>Fortress</t>
         </is>
       </c>
       <c r="AU14" s="24" t="inlineStr">
         <is>
-          <t>Mai Tai</t>
+          <t>Fortress</t>
         </is>
       </c>
       <c r="AV14" s="24" t="n"/>
@@ -5145,7 +5159,7 @@
       </c>
       <c r="BA14" s="24" t="inlineStr">
         <is>
-          <t>90a833898e793d48aa6ce23d298a692fd7b914cfa51b8101005c627e8a886f30</t>
+          <t>fd9cf8a872a6fb2106f2c32f1ebfcd0ded61283a97c1b08ceb3f2a98e39fcf6d</t>
         </is>
       </c>
       <c r="BB14" s="24" t="inlineStr">
@@ -5160,7 +5174,7 @@
       </c>
       <c r="BD14" s="24" t="inlineStr">
         <is>
-          <t>90a833898e793d48aa6ce23d298a692fd7b914cfa51b8101005c627e8a886f30</t>
+          <t>fd9cf8a872a6fb2106f2c32f1ebfcd0ded61283a97c1b08ceb3f2a98e39fcf6d</t>
         </is>
       </c>
       <c r="BE14" s="24" t="inlineStr">
@@ -5180,7 +5194,7 @@
       </c>
       <c r="BH14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T13:07:36.093507Z</t>
+          <t>2026-08-02T15:51:25.435587Z</t>
         </is>
       </c>
       <c r="BI14" s="24" t="inlineStr">
@@ -5190,13 +5204,13 @@
       </c>
       <c r="BJ14" s="25" t="n"/>
       <c r="BK14" s="26" t="n">
-        <v>-170</v>
+        <v>-156</v>
       </c>
       <c r="BL14" s="27" t="n">
-        <v>1.588235</v>
+        <v>1.641026</v>
       </c>
       <c r="BM14" s="28" t="n">
-        <v>0.62963</v>
+        <v>0.609375</v>
       </c>
       <c r="BN14" s="28" t="n"/>
       <c r="BO14" s="28" t="n"/>
@@ -5226,7 +5240,543 @@
       <c r="CM14" s="24" t="n"/>
       <c r="CN14" s="24" t="n"/>
       <c r="CO14" s="24" t="n"/>
-      <c r="CP14" s="24" t="n"/>
+      <c r="CP14" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>4a9cb06be6c94e51</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T15:51:41.323824Z</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T10:00:00Z</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>68289</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J15" s="25" t="n"/>
+      <c r="K15" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L15" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M15" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N15" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O15" s="28" t="n">
+        <v>0.599394</v>
+      </c>
+      <c r="P15" s="28" t="n"/>
+      <c r="Q15" s="28" t="n">
+        <v>0.019562</v>
+      </c>
+      <c r="R15" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="S15" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U15" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="n"/>
+      <c r="W15" s="26" t="n"/>
+      <c r="X15" s="26" t="n"/>
+      <c r="Y15" s="25" t="n"/>
+      <c r="Z15" s="26" t="n"/>
+      <c r="AA15" s="28" t="n"/>
+      <c r="AB15" s="28" t="n"/>
+      <c r="AC15" s="30" t="n"/>
+      <c r="AD15" s="24" t="n"/>
+      <c r="AE15" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF15" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG15" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH15" s="24" t="n"/>
+      <c r="AI15" s="31" t="n"/>
+      <c r="AJ15" s="31" t="n"/>
+      <c r="AK15" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL15" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM15" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN15" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO15" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AQ15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AR15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AS15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AT15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AU15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AV15" s="24" t="n"/>
+      <c r="AW15" s="24" t="n"/>
+      <c r="AX15" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY15" s="24" t="n"/>
+      <c r="AZ15" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA15" s="24" t="inlineStr">
+        <is>
+          <t>fd9cf8a872a6fb2106f2c32f1ebfcd0ded61283a97c1b08ceb3f2a98e39fcf6d</t>
+        </is>
+      </c>
+      <c r="BB15" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD15" s="24" t="inlineStr">
+        <is>
+          <t>fd9cf8a872a6fb2106f2c32f1ebfcd0ded61283a97c1b08ceb3f2a98e39fcf6d</t>
+        </is>
+      </c>
+      <c r="BE15" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF15" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T15:51:31.676274Z</t>
+        </is>
+      </c>
+      <c r="BI15" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ15" s="25" t="n"/>
+      <c r="BK15" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL15" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM15" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN15" s="28" t="n"/>
+      <c r="BO15" s="28" t="n"/>
+      <c r="BP15" s="25" t="n"/>
+      <c r="BQ15" s="27" t="n"/>
+      <c r="BR15" s="28" t="n"/>
+      <c r="BS15" s="28" t="n"/>
+      <c r="BT15" s="28" t="n"/>
+      <c r="BU15" s="25" t="n"/>
+      <c r="BV15" s="29" t="n"/>
+      <c r="BW15" s="24" t="n"/>
+      <c r="BX15" s="30" t="n"/>
+      <c r="BY15" s="27" t="n"/>
+      <c r="BZ15" s="24" t="n"/>
+      <c r="CA15" s="31" t="n"/>
+      <c r="CB15" s="24" t="n"/>
+      <c r="CC15" s="24" t="n"/>
+      <c r="CD15" s="24" t="n"/>
+      <c r="CE15" s="24" t="n"/>
+      <c r="CF15" s="24" t="n"/>
+      <c r="CG15" s="24" t="n"/>
+      <c r="CH15" s="24" t="n"/>
+      <c r="CI15" s="24" t="n"/>
+      <c r="CJ15" s="24" t="n"/>
+      <c r="CK15" s="24" t="n"/>
+      <c r="CL15" s="24" t="n"/>
+      <c r="CM15" s="24" t="n"/>
+      <c r="CN15" s="24" t="n"/>
+      <c r="CO15" s="24" t="n"/>
+      <c r="CP15" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>700b618c42d4405b</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T15:51:41.323824Z</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>69268</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M16" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N16" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O16" s="28" t="n">
+        <v>0.6819730000000001</v>
+      </c>
+      <c r="P16" s="28" t="n"/>
+      <c r="Q16" s="28" t="n">
+        <v>0.041685</v>
+      </c>
+      <c r="R16" s="26" t="n">
+        <v>41</v>
+      </c>
+      <c r="S16" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U16" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V16" s="24" t="n"/>
+      <c r="W16" s="26" t="n"/>
+      <c r="X16" s="26" t="n"/>
+      <c r="Y16" s="25" t="n"/>
+      <c r="Z16" s="26" t="n"/>
+      <c r="AA16" s="28" t="n"/>
+      <c r="AB16" s="28" t="n"/>
+      <c r="AC16" s="30" t="n"/>
+      <c r="AD16" s="24" t="n"/>
+      <c r="AE16" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF16" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG16" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH16" s="24" t="n"/>
+      <c r="AI16" s="31" t="n"/>
+      <c r="AJ16" s="31" t="n"/>
+      <c r="AK16" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL16" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN16" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AQ16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AR16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AS16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AT16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AU16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AV16" s="24" t="n"/>
+      <c r="AW16" s="24" t="n"/>
+      <c r="AX16" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY16" s="24" t="n"/>
+      <c r="AZ16" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA16" s="24" t="inlineStr">
+        <is>
+          <t>fd9cf8a872a6fb2106f2c32f1ebfcd0ded61283a97c1b08ceb3f2a98e39fcf6d</t>
+        </is>
+      </c>
+      <c r="BB16" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD16" s="24" t="inlineStr">
+        <is>
+          <t>fd9cf8a872a6fb2106f2c32f1ebfcd0ded61283a97c1b08ceb3f2a98e39fcf6d</t>
+        </is>
+      </c>
+      <c r="BE16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T15:51:37.423413Z</t>
+        </is>
+      </c>
+      <c r="BI16" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ16" s="25" t="n"/>
+      <c r="BK16" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL16" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM16" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN16" s="28" t="n"/>
+      <c r="BO16" s="28" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
+      <c r="BR16" s="28" t="n"/>
+      <c r="BS16" s="28" t="n"/>
+      <c r="BT16" s="28" t="n"/>
+      <c r="BU16" s="25" t="n"/>
+      <c r="BV16" s="29" t="n"/>
+      <c r="BW16" s="24" t="n"/>
+      <c r="BX16" s="30" t="n"/>
+      <c r="BY16" s="27" t="n"/>
+      <c r="BZ16" s="24" t="n"/>
+      <c r="CA16" s="31" t="n"/>
+      <c r="CB16" s="24" t="n"/>
+      <c r="CC16" s="24" t="n"/>
+      <c r="CD16" s="24" t="n"/>
+      <c r="CE16" s="24" t="n"/>
+      <c r="CF16" s="24" t="n"/>
+      <c r="CG16" s="24" t="n"/>
+      <c r="CH16" s="24" t="n"/>
+      <c r="CI16" s="24" t="n"/>
+      <c r="CJ16" s="24" t="n"/>
+      <c r="CK16" s="24" t="n"/>
+      <c r="CL16" s="24" t="n"/>
+      <c r="CM16" s="24" t="n"/>
+      <c r="CN16" s="24" t="n"/>
+      <c r="CO16" s="24" t="n"/>
+      <c r="CP16" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: P1-17 MLB totals over-selection bias root-cause investigation (Claude)
Root-caused via live code + real ledger data: weak elasticities (offense/park/weather/starter all << 1.0) cause near-constant per-game run projections, plus selection happening pre-calibration in forward.py. 71% over-picked, overs 30% hit rate vs unders 55%. Flat-only/zero-unit so no real capital at risk. Fix requires real elasticity refit against totals outcomes specifically — cross-referenced in MLB roadmap item 5. Includes pipeline data and config/model sync from 2026-08-03 session.
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ15" headerRowCount="1">
-  <autoFilter ref="A1:CQ15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ16" headerRowCount="1">
+  <autoFilter ref="A1:CQ16"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$15)</f>
+        <f>COUNTA('Picks'!$A$2:$A$16)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$15,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$16,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")+COUNTIFS('Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$15,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$16,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"win")/(COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"win")+COUNTIFS('Picks'!$BX$2:$BX$15,"&gt;0",'Picks'!$V$2:$V$15,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")/(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$15)/SUM('Picks'!$BX$2:$BX$15),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$16)/SUM('Picks'!$BX$2:$BX$16),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$15)</f>
+        <f>SUM('Picks'!$BY$2:$BY$16)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$15,"&lt;&gt;",'Picks'!$AB$2:$AB$15),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$16,"&lt;&gt;",'Picks'!$AB$2:$AB$16),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$15,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$15,'Picks'!$AM$2:$AM$15,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$16,'Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$15,'Picks'!$H$2:$H$15,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$15,'Picks'!$H$2:$H$15,$A14,'Picks'!$U$2:$U$15,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$15,'Picks'!$H$2:$H$15,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$15,'Picks'!$H$2:$H$15,$A15,'Picks'!$U$2:$U$15,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled",'Picks'!$V$2:$V$15,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$15,'Picks'!$H$2:$H$15,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$15,'Picks'!$H$2:$H$15,$A16,'Picks'!$U$2:$U$15,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ15"/>
+  <dimension ref="A1:CQ16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5002,22 +5002,22 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>a975e837b88c43d8</t>
+          <t>d46b1c6c074d4d79</t>
         </is>
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T16:15:14.476529Z</t>
+          <t>2026-08-02T16:53:33.678893Z</t>
         </is>
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-03T10:00:00Z</t>
+          <t>2026-08-02T17:00:00Z</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>68289</t>
+          <t>69263</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
@@ -5027,12 +5027,12 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="H14" s="24" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J14" s="25" t="n"/>
@@ -5052,26 +5052,26 @@
         </is>
       </c>
       <c r="L14" s="26" t="n">
-        <v>-138</v>
+        <v>-194</v>
       </c>
       <c r="M14" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.515464</v>
       </c>
       <c r="N14" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.659864</v>
       </c>
       <c r="O14" s="28" t="n">
-        <v>0.599195</v>
+        <v>0.68024</v>
       </c>
       <c r="P14" s="28" t="n"/>
       <c r="Q14" s="28" t="n">
-        <v>0.019363</v>
+        <v>0.020376</v>
       </c>
       <c r="R14" s="26" t="n">
         <v>30</v>
       </c>
       <c r="S14" s="29" t="n">
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="T14" s="24" t="inlineStr">
         <is>
@@ -5094,7 +5094,7 @@
       <c r="AD14" s="24" t="n"/>
       <c r="AE14" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
+          <t>Neutral Elo baseline; executable ask 0.6600 (market_slug=aec-cs2-mta-enjoy-2026-08-02).</t>
         </is>
       </c>
       <c r="AF14" s="31" t="inlineStr">
@@ -5135,32 +5135,32 @@
       </c>
       <c r="AP14" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="AQ14" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="AR14" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>ENJOY</t>
         </is>
       </c>
       <c r="AS14" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="AT14" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="AU14" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>Mai Tai</t>
         </is>
       </c>
       <c r="AV14" s="24" t="n"/>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="BA14" s="24" t="inlineStr">
         <is>
-          <t>be57084f1d7fbd4d502df5071cd07ad0aef0fe46ec9ff6b18e470efb3b2bbfd4</t>
+          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
         </is>
       </c>
       <c r="BB14" s="24" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="BD14" s="24" t="inlineStr">
         <is>
-          <t>be57084f1d7fbd4d502df5071cd07ad0aef0fe46ec9ff6b18e470efb3b2bbfd4</t>
+          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
         </is>
       </c>
       <c r="BE14" s="24" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="BH14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T16:15:04.678326Z</t>
+          <t>2026-08-02T16:53:19.829844Z</t>
         </is>
       </c>
       <c r="BI14" s="24" t="inlineStr">
@@ -5223,13 +5223,13 @@
       </c>
       <c r="BJ14" s="25" t="n"/>
       <c r="BK14" s="26" t="n">
-        <v>-138</v>
+        <v>-194</v>
       </c>
       <c r="BL14" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.515464</v>
       </c>
       <c r="BM14" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.659864</v>
       </c>
       <c r="BN14" s="28" t="n"/>
       <c r="BO14" s="28" t="n"/>
@@ -5269,22 +5269,22 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>4c4413651a2a4ceb</t>
+          <t>b0445f7352d444ff</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T16:15:14.476529Z</t>
+          <t>2026-08-02T16:53:33.678893Z</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-03T14:00:00Z</t>
+          <t>2026-08-03T10:00:00Z</t>
         </is>
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>69268</t>
+          <t>68289</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
@@ -5294,12 +5294,12 @@
       </c>
       <c r="F15" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>FURY</t>
         </is>
       </c>
       <c r="G15" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Mindfreak</t>
         </is>
       </c>
       <c r="H15" s="24" t="inlineStr">
@@ -5319,26 +5319,26 @@
         </is>
       </c>
       <c r="L15" s="26" t="n">
-        <v>-178</v>
+        <v>-138</v>
       </c>
       <c r="M15" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.724638</v>
       </c>
       <c r="N15" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.579832</v>
       </c>
       <c r="O15" s="28" t="n">
-        <v>0.662883</v>
+        <v>0.599198</v>
       </c>
       <c r="P15" s="28" t="n"/>
       <c r="Q15" s="28" t="n">
-        <v>0.022595</v>
+        <v>0.019366</v>
       </c>
       <c r="R15" s="26" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S15" s="29" t="n">
-        <v>1.75</v>
+        <v>1.25</v>
       </c>
       <c r="T15" s="24" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
       <c r="AD15" s="24" t="n"/>
       <c r="AE15" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
         </is>
       </c>
       <c r="AF15" s="31" t="inlineStr">
@@ -5402,32 +5402,32 @@
       </c>
       <c r="AP15" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>FURY</t>
         </is>
       </c>
       <c r="AQ15" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>FURY</t>
         </is>
       </c>
       <c r="AR15" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>FURY</t>
         </is>
       </c>
       <c r="AS15" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Mindfreak</t>
         </is>
       </c>
       <c r="AT15" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Mindfreak</t>
         </is>
       </c>
       <c r="AU15" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Mindfreak</t>
         </is>
       </c>
       <c r="AV15" s="24" t="n"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="BA15" s="24" t="inlineStr">
         <is>
-          <t>be57084f1d7fbd4d502df5071cd07ad0aef0fe46ec9ff6b18e470efb3b2bbfd4</t>
+          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
         </is>
       </c>
       <c r="BB15" s="24" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="BD15" s="24" t="inlineStr">
         <is>
-          <t>be57084f1d7fbd4d502df5071cd07ad0aef0fe46ec9ff6b18e470efb3b2bbfd4</t>
+          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
         </is>
       </c>
       <c r="BE15" s="24" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="BH15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T16:15:10.799851Z</t>
+          <t>2026-08-02T16:53:25.545768Z</t>
         </is>
       </c>
       <c r="BI15" s="24" t="inlineStr">
@@ -5490,13 +5490,13 @@
       </c>
       <c r="BJ15" s="25" t="n"/>
       <c r="BK15" s="26" t="n">
-        <v>-178</v>
+        <v>-138</v>
       </c>
       <c r="BL15" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.724638</v>
       </c>
       <c r="BM15" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.579832</v>
       </c>
       <c r="BN15" s="28" t="n"/>
       <c r="BO15" s="28" t="n"/>
@@ -5533,6 +5533,273 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>0797e5dac5e74572</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T16:53:33.678893Z</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>69268</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M16" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N16" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O16" s="28" t="n">
+        <v>0.663025</v>
+      </c>
+      <c r="P16" s="28" t="n"/>
+      <c r="Q16" s="28" t="n">
+        <v>0.022737</v>
+      </c>
+      <c r="R16" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="S16" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U16" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V16" s="24" t="n"/>
+      <c r="W16" s="26" t="n"/>
+      <c r="X16" s="26" t="n"/>
+      <c r="Y16" s="25" t="n"/>
+      <c r="Z16" s="26" t="n"/>
+      <c r="AA16" s="28" t="n"/>
+      <c r="AB16" s="28" t="n"/>
+      <c r="AC16" s="30" t="n"/>
+      <c r="AD16" s="24" t="n"/>
+      <c r="AE16" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF16" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG16" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH16" s="24" t="n"/>
+      <c r="AI16" s="31" t="n"/>
+      <c r="AJ16" s="31" t="n"/>
+      <c r="AK16" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL16" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN16" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AQ16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AR16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AS16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AT16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AU16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AV16" s="24" t="n"/>
+      <c r="AW16" s="24" t="n"/>
+      <c r="AX16" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY16" s="24" t="n"/>
+      <c r="AZ16" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA16" s="24" t="inlineStr">
+        <is>
+          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
+        </is>
+      </c>
+      <c r="BB16" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD16" s="24" t="inlineStr">
+        <is>
+          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
+        </is>
+      </c>
+      <c r="BE16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T16:53:29.527479Z</t>
+        </is>
+      </c>
+      <c r="BI16" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ16" s="25" t="n"/>
+      <c r="BK16" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL16" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM16" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN16" s="28" t="n"/>
+      <c r="BO16" s="28" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
+      <c r="BR16" s="28" t="n"/>
+      <c r="BS16" s="28" t="n"/>
+      <c r="BT16" s="28" t="n"/>
+      <c r="BU16" s="25" t="n"/>
+      <c r="BV16" s="29" t="n"/>
+      <c r="BW16" s="24" t="n"/>
+      <c r="BX16" s="30" t="n"/>
+      <c r="BY16" s="27" t="n"/>
+      <c r="BZ16" s="24" t="n"/>
+      <c r="CA16" s="31" t="n"/>
+      <c r="CB16" s="24" t="n"/>
+      <c r="CC16" s="24" t="n"/>
+      <c r="CD16" s="24" t="n"/>
+      <c r="CE16" s="24" t="n"/>
+      <c r="CF16" s="24" t="n"/>
+      <c r="CG16" s="24" t="n"/>
+      <c r="CH16" s="24" t="n"/>
+      <c r="CI16" s="24" t="n"/>
+      <c r="CJ16" s="24" t="n"/>
+      <c r="CK16" s="24" t="n"/>
+      <c r="CL16" s="24" t="n"/>
+      <c r="CM16" s="24" t="n"/>
+      <c r="CN16" s="24" t="n"/>
+      <c r="CO16" s="24" t="n"/>
+      <c r="CP16" s="24" t="n"/>
+      <c r="CQ16" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix: Main ledger gated-only, _forecast_mlb_totals_flat Main writes now CALL-gated, 654 tests pass
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ16" headerRowCount="1">
-  <autoFilter ref="A1:CQ16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ14" headerRowCount="1">
+  <autoFilter ref="A1:CQ14"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$16)</f>
+        <f>COUNTA('Picks'!$A$2:$A$14)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$16,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$16,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")/(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$16)/SUM('Picks'!$BX$2:$BX$16),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$16)</f>
+        <f>SUM('Picks'!$BY$2:$BY$14)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$16,"&lt;&gt;",'Picks'!$AB$2:$AB$16),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$16,'Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ16"/>
+  <dimension ref="A1:CQ14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5266,540 +5266,6 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>b0445f7352d444ff</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:33.678893Z</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T10:00:00Z</t>
-        </is>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>68289</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="G15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="H15" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I15" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J15" s="25" t="n"/>
-      <c r="K15" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L15" s="26" t="n">
-        <v>-138</v>
-      </c>
-      <c r="M15" s="27" t="n">
-        <v>1.724638</v>
-      </c>
-      <c r="N15" s="28" t="n">
-        <v>0.579832</v>
-      </c>
-      <c r="O15" s="28" t="n">
-        <v>0.599198</v>
-      </c>
-      <c r="P15" s="28" t="n"/>
-      <c r="Q15" s="28" t="n">
-        <v>0.019366</v>
-      </c>
-      <c r="R15" s="26" t="n">
-        <v>30</v>
-      </c>
-      <c r="S15" s="29" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="T15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U15" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V15" s="24" t="n"/>
-      <c r="W15" s="26" t="n"/>
-      <c r="X15" s="26" t="n"/>
-      <c r="Y15" s="25" t="n"/>
-      <c r="Z15" s="26" t="n"/>
-      <c r="AA15" s="28" t="n"/>
-      <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n"/>
-      <c r="AD15" s="24" t="n"/>
-      <c r="AE15" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF15" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG15" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH15" s="24" t="n"/>
-      <c r="AI15" s="31" t="n"/>
-      <c r="AJ15" s="31" t="n"/>
-      <c r="AK15" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL15" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM15" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN15" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO15" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="AQ15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="AR15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="AS15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="AT15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="AU15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="AV15" s="24" t="n"/>
-      <c r="AW15" s="24" t="n"/>
-      <c r="AX15" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY15" s="24" t="n"/>
-      <c r="AZ15" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA15" s="24" t="inlineStr">
-        <is>
-          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
-        </is>
-      </c>
-      <c r="BB15" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD15" s="24" t="inlineStr">
-        <is>
-          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
-        </is>
-      </c>
-      <c r="BE15" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF15" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:25.545768Z</t>
-        </is>
-      </c>
-      <c r="BI15" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ15" s="25" t="n"/>
-      <c r="BK15" s="26" t="n">
-        <v>-138</v>
-      </c>
-      <c r="BL15" s="27" t="n">
-        <v>1.724638</v>
-      </c>
-      <c r="BM15" s="28" t="n">
-        <v>0.579832</v>
-      </c>
-      <c r="BN15" s="28" t="n"/>
-      <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
-      <c r="BR15" s="28" t="n"/>
-      <c r="BS15" s="28" t="n"/>
-      <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="25" t="n"/>
-      <c r="BV15" s="29" t="n"/>
-      <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="30" t="n"/>
-      <c r="BY15" s="27" t="n"/>
-      <c r="BZ15" s="24" t="n"/>
-      <c r="CA15" s="31" t="n"/>
-      <c r="CB15" s="24" t="n"/>
-      <c r="CC15" s="24" t="n"/>
-      <c r="CD15" s="24" t="n"/>
-      <c r="CE15" s="24" t="n"/>
-      <c r="CF15" s="24" t="n"/>
-      <c r="CG15" s="24" t="n"/>
-      <c r="CH15" s="24" t="n"/>
-      <c r="CI15" s="24" t="n"/>
-      <c r="CJ15" s="24" t="n"/>
-      <c r="CK15" s="24" t="n"/>
-      <c r="CL15" s="24" t="n"/>
-      <c r="CM15" s="24" t="n"/>
-      <c r="CN15" s="24" t="n"/>
-      <c r="CO15" s="24" t="n"/>
-      <c r="CP15" s="24" t="n"/>
-      <c r="CQ15" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>0797e5dac5e74572</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:33.678893Z</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T14:00:00Z</t>
-        </is>
-      </c>
-      <c r="D16" s="24" t="inlineStr">
-        <is>
-          <t>69268</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="G16" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="H16" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I16" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J16" s="25" t="n"/>
-      <c r="K16" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L16" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="M16" s="27" t="n">
-        <v>1.561798</v>
-      </c>
-      <c r="N16" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="O16" s="28" t="n">
-        <v>0.663025</v>
-      </c>
-      <c r="P16" s="28" t="n"/>
-      <c r="Q16" s="28" t="n">
-        <v>0.022737</v>
-      </c>
-      <c r="R16" s="26" t="n">
-        <v>31</v>
-      </c>
-      <c r="S16" s="29" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="T16" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U16" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V16" s="24" t="n"/>
-      <c r="W16" s="26" t="n"/>
-      <c r="X16" s="26" t="n"/>
-      <c r="Y16" s="25" t="n"/>
-      <c r="Z16" s="26" t="n"/>
-      <c r="AA16" s="28" t="n"/>
-      <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="30" t="n"/>
-      <c r="AD16" s="24" t="n"/>
-      <c r="AE16" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF16" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG16" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH16" s="24" t="n"/>
-      <c r="AI16" s="31" t="n"/>
-      <c r="AJ16" s="31" t="n"/>
-      <c r="AK16" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL16" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM16" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN16" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO16" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP16" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="AQ16" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="AR16" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="AS16" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="AT16" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="AU16" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="AV16" s="24" t="n"/>
-      <c r="AW16" s="24" t="n"/>
-      <c r="AX16" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY16" s="24" t="n"/>
-      <c r="AZ16" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA16" s="24" t="inlineStr">
-        <is>
-          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
-        </is>
-      </c>
-      <c r="BB16" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC16" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD16" s="24" t="inlineStr">
-        <is>
-          <t>4c897e659ec9db491c18706ace7c94ba8af6df222c16d377d3bd7391aba18f91</t>
-        </is>
-      </c>
-      <c r="BE16" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF16" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG16" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH16" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:29.527479Z</t>
-        </is>
-      </c>
-      <c r="BI16" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ16" s="25" t="n"/>
-      <c r="BK16" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="BL16" s="27" t="n">
-        <v>1.561798</v>
-      </c>
-      <c r="BM16" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="BN16" s="28" t="n"/>
-      <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="25" t="n"/>
-      <c r="BQ16" s="27" t="n"/>
-      <c r="BR16" s="28" t="n"/>
-      <c r="BS16" s="28" t="n"/>
-      <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="25" t="n"/>
-      <c r="BV16" s="29" t="n"/>
-      <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="30" t="n"/>
-      <c r="BY16" s="27" t="n"/>
-      <c r="BZ16" s="24" t="n"/>
-      <c r="CA16" s="31" t="n"/>
-      <c r="CB16" s="24" t="n"/>
-      <c r="CC16" s="24" t="n"/>
-      <c r="CD16" s="24" t="n"/>
-      <c r="CE16" s="24" t="n"/>
-      <c r="CF16" s="24" t="n"/>
-      <c r="CG16" s="24" t="n"/>
-      <c r="CH16" s="24" t="n"/>
-      <c r="CI16" s="24" t="n"/>
-      <c r="CJ16" s="24" t="n"/>
-      <c r="CK16" s="24" t="n"/>
-      <c r="CL16" s="24" t="n"/>
-      <c r="CM16" s="24" t="n"/>
-      <c r="CN16" s="24" t="n"/>
-      <c r="CO16" s="24" t="n"/>
-      <c r="CP16" s="24" t="n"/>
-      <c r="CQ16" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix: research_ledger default=None in soccer/tennis forecast, docs: LEDGER_ROUTING.md rewritten, daily pipeline data sync, 654 tests pass
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ14" headerRowCount="1">
-  <autoFilter ref="A1:CQ14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ16" headerRowCount="1">
+  <autoFilter ref="A1:CQ16"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$14)</f>
+        <f>COUNTA('Picks'!$A$2:$A$16)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$16,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$16,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")/(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$16)/SUM('Picks'!$BX$2:$BX$16),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$14)</f>
+        <f>SUM('Picks'!$BY$2:$BY$16)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$16,"&lt;&gt;",'Picks'!$AB$2:$AB$16),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$16,'Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ14"/>
+  <dimension ref="A1:CQ16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5266,6 +5266,540 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>527b87d97fca4de2</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T17:48:41.505470Z</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T10:00:00Z</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>68289</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J15" s="25" t="n"/>
+      <c r="K15" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L15" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M15" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N15" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O15" s="28" t="n">
+        <v>0.599199</v>
+      </c>
+      <c r="P15" s="28" t="n"/>
+      <c r="Q15" s="28" t="n">
+        <v>0.019367</v>
+      </c>
+      <c r="R15" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="S15" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U15" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="n"/>
+      <c r="W15" s="26" t="n"/>
+      <c r="X15" s="26" t="n"/>
+      <c r="Y15" s="25" t="n"/>
+      <c r="Z15" s="26" t="n"/>
+      <c r="AA15" s="28" t="n"/>
+      <c r="AB15" s="28" t="n"/>
+      <c r="AC15" s="30" t="n"/>
+      <c r="AD15" s="24" t="n"/>
+      <c r="AE15" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF15" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG15" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH15" s="24" t="n"/>
+      <c r="AI15" s="31" t="n"/>
+      <c r="AJ15" s="31" t="n"/>
+      <c r="AK15" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL15" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM15" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN15" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO15" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AQ15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AR15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AS15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AT15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AU15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AV15" s="24" t="n"/>
+      <c r="AW15" s="24" t="n"/>
+      <c r="AX15" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY15" s="24" t="n"/>
+      <c r="AZ15" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA15" s="24" t="inlineStr">
+        <is>
+          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+        </is>
+      </c>
+      <c r="BB15" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD15" s="24" t="inlineStr">
+        <is>
+          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+        </is>
+      </c>
+      <c r="BE15" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF15" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T17:48:31.821007Z</t>
+        </is>
+      </c>
+      <c r="BI15" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ15" s="25" t="n"/>
+      <c r="BK15" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL15" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM15" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN15" s="28" t="n"/>
+      <c r="BO15" s="28" t="n"/>
+      <c r="BP15" s="25" t="n"/>
+      <c r="BQ15" s="27" t="n"/>
+      <c r="BR15" s="28" t="n"/>
+      <c r="BS15" s="28" t="n"/>
+      <c r="BT15" s="28" t="n"/>
+      <c r="BU15" s="25" t="n"/>
+      <c r="BV15" s="29" t="n"/>
+      <c r="BW15" s="24" t="n"/>
+      <c r="BX15" s="30" t="n"/>
+      <c r="BY15" s="27" t="n"/>
+      <c r="BZ15" s="24" t="n"/>
+      <c r="CA15" s="31" t="n"/>
+      <c r="CB15" s="24" t="n"/>
+      <c r="CC15" s="24" t="n"/>
+      <c r="CD15" s="24" t="n"/>
+      <c r="CE15" s="24" t="n"/>
+      <c r="CF15" s="24" t="n"/>
+      <c r="CG15" s="24" t="n"/>
+      <c r="CH15" s="24" t="n"/>
+      <c r="CI15" s="24" t="n"/>
+      <c r="CJ15" s="24" t="n"/>
+      <c r="CK15" s="24" t="n"/>
+      <c r="CL15" s="24" t="n"/>
+      <c r="CM15" s="24" t="n"/>
+      <c r="CN15" s="24" t="n"/>
+      <c r="CO15" s="24" t="n"/>
+      <c r="CP15" s="24" t="n"/>
+      <c r="CQ15" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>50897d877f614f10</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T17:48:41.505470Z</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>69268</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M16" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N16" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O16" s="28" t="n">
+        <v>0.663041</v>
+      </c>
+      <c r="P16" s="28" t="n"/>
+      <c r="Q16" s="28" t="n">
+        <v>0.022753</v>
+      </c>
+      <c r="R16" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="S16" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U16" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V16" s="24" t="n"/>
+      <c r="W16" s="26" t="n"/>
+      <c r="X16" s="26" t="n"/>
+      <c r="Y16" s="25" t="n"/>
+      <c r="Z16" s="26" t="n"/>
+      <c r="AA16" s="28" t="n"/>
+      <c r="AB16" s="28" t="n"/>
+      <c r="AC16" s="30" t="n"/>
+      <c r="AD16" s="24" t="n"/>
+      <c r="AE16" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF16" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG16" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH16" s="24" t="n"/>
+      <c r="AI16" s="31" t="n"/>
+      <c r="AJ16" s="31" t="n"/>
+      <c r="AK16" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL16" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN16" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AQ16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AR16" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AS16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AT16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AU16" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AV16" s="24" t="n"/>
+      <c r="AW16" s="24" t="n"/>
+      <c r="AX16" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY16" s="24" t="n"/>
+      <c r="AZ16" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA16" s="24" t="inlineStr">
+        <is>
+          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+        </is>
+      </c>
+      <c r="BB16" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD16" s="24" t="inlineStr">
+        <is>
+          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+        </is>
+      </c>
+      <c r="BE16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T17:48:36.924167Z</t>
+        </is>
+      </c>
+      <c r="BI16" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ16" s="25" t="n"/>
+      <c r="BK16" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL16" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM16" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN16" s="28" t="n"/>
+      <c r="BO16" s="28" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
+      <c r="BR16" s="28" t="n"/>
+      <c r="BS16" s="28" t="n"/>
+      <c r="BT16" s="28" t="n"/>
+      <c r="BU16" s="25" t="n"/>
+      <c r="BV16" s="29" t="n"/>
+      <c r="BW16" s="24" t="n"/>
+      <c r="BX16" s="30" t="n"/>
+      <c r="BY16" s="27" t="n"/>
+      <c r="BZ16" s="24" t="n"/>
+      <c r="CA16" s="31" t="n"/>
+      <c r="CB16" s="24" t="n"/>
+      <c r="CC16" s="24" t="n"/>
+      <c r="CD16" s="24" t="n"/>
+      <c r="CE16" s="24" t="n"/>
+      <c r="CF16" s="24" t="n"/>
+      <c r="CG16" s="24" t="n"/>
+      <c r="CH16" s="24" t="n"/>
+      <c r="CI16" s="24" t="n"/>
+      <c r="CJ16" s="24" t="n"/>
+      <c r="CK16" s="24" t="n"/>
+      <c r="CL16" s="24" t="n"/>
+      <c r="CM16" s="24" t="n"/>
+      <c r="CN16" s="24" t="n"/>
+      <c r="CO16" s="24" t="n"/>
+      <c r="CP16" s="24" t="n"/>
+      <c r="CQ16" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
chore: MASTER.md update, pipeline data sync, 654 tests pass
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ16" headerRowCount="1">
-  <autoFilter ref="A1:CQ16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ17" headerRowCount="1">
+  <autoFilter ref="A1:CQ17"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$16)</f>
+        <f>COUNTA('Picks'!$A$2:$A$17)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$16,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$17,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$16,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$17,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")/(COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"win")+COUNTIFS('Picks'!$BX$2:$BX$16,"&gt;0",'Picks'!$V$2:$V$16,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")/(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$16)/SUM('Picks'!$BX$2:$BX$16),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$17)/SUM('Picks'!$BX$2:$BX$17),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$16)</f>
+        <f>SUM('Picks'!$BY$2:$BY$17)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$16,"&lt;&gt;",'Picks'!$AB$2:$AB$16),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$17,"&lt;&gt;",'Picks'!$AB$2:$AB$17),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$16,'Picks'!$AM$2:$AM$16,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$17,'Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A14,'Picks'!$U$2:$U$16,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A15,'Picks'!$U$2:$U$16,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled",'Picks'!$V$2:$V$16,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$16,'Picks'!$H$2:$H$16,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$16,'Picks'!$H$2:$H$16,$A16,'Picks'!$U$2:$U$16,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ16"/>
+  <dimension ref="A1:CQ17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5269,12 +5269,12 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>527b87d97fca4de2</t>
+          <t>936b606e7d544e3c</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T17:48:41.505470Z</t>
+          <t>2026-08-02T18:08:55.998248Z</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="BA15" s="24" t="inlineStr">
         <is>
-          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
         </is>
       </c>
       <c r="BB15" s="24" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="BD15" s="24" t="inlineStr">
         <is>
-          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
         </is>
       </c>
       <c r="BE15" s="24" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="BH15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T17:48:31.821007Z</t>
+          <t>2026-08-02T18:08:46.352076Z</t>
         </is>
       </c>
       <c r="BI15" s="24" t="inlineStr">
@@ -5536,22 +5536,22 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>50897d877f614f10</t>
+          <t>db1dc943d75f40cf</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T17:48:41.505470Z</t>
+          <t>2026-08-02T18:08:55.998248Z</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-03T14:00:00Z</t>
+          <t>2026-08-03T10:30:00Z</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>69268</t>
+          <t>67514</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
@@ -5561,12 +5561,12 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="H16" s="24" t="inlineStr">
@@ -5586,26 +5586,26 @@
         </is>
       </c>
       <c r="L16" s="26" t="n">
-        <v>-178</v>
+        <v>-163</v>
       </c>
       <c r="M16" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.613497</v>
       </c>
       <c r="N16" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.619772</v>
       </c>
       <c r="O16" s="28" t="n">
-        <v>0.663041</v>
+        <v>0.639896</v>
       </c>
       <c r="P16" s="28" t="n"/>
       <c r="Q16" s="28" t="n">
-        <v>0.022753</v>
+        <v>0.020124</v>
       </c>
       <c r="R16" s="26" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S16" s="29" t="n">
-        <v>1.75</v>
+        <v>1.5</v>
       </c>
       <c r="T16" s="24" t="inlineStr">
         <is>
@@ -5628,7 +5628,7 @@
       <c r="AD16" s="24" t="n"/>
       <c r="AE16" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-cs2-era-psna-2026-08-03).</t>
         </is>
       </c>
       <c r="AF16" s="31" t="inlineStr">
@@ -5669,32 +5669,32 @@
       </c>
       <c r="AP16" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="AQ16" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="AR16" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="AS16" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="AT16" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="AU16" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="AV16" s="24" t="n"/>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="BA16" s="24" t="inlineStr">
         <is>
-          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
         </is>
       </c>
       <c r="BB16" s="24" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="BD16" s="24" t="inlineStr">
         <is>
-          <t>a4e21a1af368f0354dc5f9a4308bc7027cac0942d4270c2251f9210a7793ef91</t>
+          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
         </is>
       </c>
       <c r="BE16" s="24" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="BH16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T17:48:36.924167Z</t>
+          <t>2026-08-02T18:08:48.789246Z</t>
         </is>
       </c>
       <c r="BI16" s="24" t="inlineStr">
@@ -5757,13 +5757,13 @@
       </c>
       <c r="BJ16" s="25" t="n"/>
       <c r="BK16" s="26" t="n">
-        <v>-178</v>
+        <v>-163</v>
       </c>
       <c r="BL16" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.613497</v>
       </c>
       <c r="BM16" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.619772</v>
       </c>
       <c r="BN16" s="28" t="n"/>
       <c r="BO16" s="28" t="n"/>
@@ -5800,6 +5800,273 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>d60a6e820d4f4adc</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:08:55.998248Z</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>69268</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J17" s="25" t="n"/>
+      <c r="K17" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M17" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N17" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O17" s="28" t="n">
+        <v>0.663041</v>
+      </c>
+      <c r="P17" s="28" t="n"/>
+      <c r="Q17" s="28" t="n">
+        <v>0.022753</v>
+      </c>
+      <c r="R17" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="S17" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T17" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U17" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V17" s="24" t="n"/>
+      <c r="W17" s="26" t="n"/>
+      <c r="X17" s="26" t="n"/>
+      <c r="Y17" s="25" t="n"/>
+      <c r="Z17" s="26" t="n"/>
+      <c r="AA17" s="28" t="n"/>
+      <c r="AB17" s="28" t="n"/>
+      <c r="AC17" s="30" t="n"/>
+      <c r="AD17" s="24" t="n"/>
+      <c r="AE17" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF17" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG17" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH17" s="24" t="n"/>
+      <c r="AI17" s="31" t="n"/>
+      <c r="AJ17" s="31" t="n"/>
+      <c r="AK17" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL17" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM17" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN17" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO17" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AQ17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AR17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AS17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AT17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AU17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AV17" s="24" t="n"/>
+      <c r="AW17" s="24" t="n"/>
+      <c r="AX17" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY17" s="24" t="n"/>
+      <c r="AZ17" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA17" s="24" t="inlineStr">
+        <is>
+          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
+        </is>
+      </c>
+      <c r="BB17" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC17" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD17" s="24" t="inlineStr">
+        <is>
+          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
+        </is>
+      </c>
+      <c r="BE17" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF17" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG17" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH17" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:08:51.418739Z</t>
+        </is>
+      </c>
+      <c r="BI17" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ17" s="25" t="n"/>
+      <c r="BK17" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL17" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM17" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN17" s="28" t="n"/>
+      <c r="BO17" s="28" t="n"/>
+      <c r="BP17" s="25" t="n"/>
+      <c r="BQ17" s="27" t="n"/>
+      <c r="BR17" s="28" t="n"/>
+      <c r="BS17" s="28" t="n"/>
+      <c r="BT17" s="28" t="n"/>
+      <c r="BU17" s="25" t="n"/>
+      <c r="BV17" s="29" t="n"/>
+      <c r="BW17" s="24" t="n"/>
+      <c r="BX17" s="30" t="n"/>
+      <c r="BY17" s="27" t="n"/>
+      <c r="BZ17" s="24" t="n"/>
+      <c r="CA17" s="31" t="n"/>
+      <c r="CB17" s="24" t="n"/>
+      <c r="CC17" s="24" t="n"/>
+      <c r="CD17" s="24" t="n"/>
+      <c r="CE17" s="24" t="n"/>
+      <c r="CF17" s="24" t="n"/>
+      <c r="CG17" s="24" t="n"/>
+      <c r="CH17" s="24" t="n"/>
+      <c r="CI17" s="24" t="n"/>
+      <c r="CJ17" s="24" t="n"/>
+      <c r="CK17" s="24" t="n"/>
+      <c r="CL17" s="24" t="n"/>
+      <c r="CM17" s="24" t="n"/>
+      <c r="CN17" s="24" t="n"/>
+      <c r="CO17" s="24" t="n"/>
+      <c r="CP17" s="24" t="n"/>
+      <c r="CQ17" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix: P1-17 MLB totals over-selection bias — calibrate before selection in forward.py, bump elasticities, clean 30 stale .bak files, 654 tests pass
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ17" headerRowCount="1">
-  <autoFilter ref="A1:CQ17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ14" headerRowCount="1">
+  <autoFilter ref="A1:CQ14"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$17)</f>
+        <f>COUNTA('Picks'!$A$2:$A$14)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$17,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$17,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")/(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$17)/SUM('Picks'!$BX$2:$BX$17),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$17)</f>
+        <f>SUM('Picks'!$BY$2:$BY$14)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$17,"&lt;&gt;",'Picks'!$AB$2:$AB$17),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$17,'Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ17"/>
+  <dimension ref="A1:CQ14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5266,807 +5266,6 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>936b606e7d544e3c</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T18:08:55.998248Z</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T10:00:00Z</t>
-        </is>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>68289</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="G15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="H15" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I15" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J15" s="25" t="n"/>
-      <c r="K15" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L15" s="26" t="n">
-        <v>-138</v>
-      </c>
-      <c r="M15" s="27" t="n">
-        <v>1.724638</v>
-      </c>
-      <c r="N15" s="28" t="n">
-        <v>0.579832</v>
-      </c>
-      <c r="O15" s="28" t="n">
-        <v>0.599199</v>
-      </c>
-      <c r="P15" s="28" t="n"/>
-      <c r="Q15" s="28" t="n">
-        <v>0.019367</v>
-      </c>
-      <c r="R15" s="26" t="n">
-        <v>30</v>
-      </c>
-      <c r="S15" s="29" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="T15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U15" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V15" s="24" t="n"/>
-      <c r="W15" s="26" t="n"/>
-      <c r="X15" s="26" t="n"/>
-      <c r="Y15" s="25" t="n"/>
-      <c r="Z15" s="26" t="n"/>
-      <c r="AA15" s="28" t="n"/>
-      <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n"/>
-      <c r="AD15" s="24" t="n"/>
-      <c r="AE15" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF15" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG15" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH15" s="24" t="n"/>
-      <c r="AI15" s="31" t="n"/>
-      <c r="AJ15" s="31" t="n"/>
-      <c r="AK15" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL15" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM15" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN15" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO15" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="AQ15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="AR15" s="24" t="inlineStr">
-        <is>
-          <t>FURY</t>
-        </is>
-      </c>
-      <c r="AS15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="AT15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="AU15" s="24" t="inlineStr">
-        <is>
-          <t>Mindfreak</t>
-        </is>
-      </c>
-      <c r="AV15" s="24" t="n"/>
-      <c r="AW15" s="24" t="n"/>
-      <c r="AX15" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY15" s="24" t="n"/>
-      <c r="AZ15" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA15" s="24" t="inlineStr">
-        <is>
-          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
-        </is>
-      </c>
-      <c r="BB15" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD15" s="24" t="inlineStr">
-        <is>
-          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
-        </is>
-      </c>
-      <c r="BE15" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF15" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG15" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH15" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T18:08:46.352076Z</t>
-        </is>
-      </c>
-      <c r="BI15" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ15" s="25" t="n"/>
-      <c r="BK15" s="26" t="n">
-        <v>-138</v>
-      </c>
-      <c r="BL15" s="27" t="n">
-        <v>1.724638</v>
-      </c>
-      <c r="BM15" s="28" t="n">
-        <v>0.579832</v>
-      </c>
-      <c r="BN15" s="28" t="n"/>
-      <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
-      <c r="BR15" s="28" t="n"/>
-      <c r="BS15" s="28" t="n"/>
-      <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="25" t="n"/>
-      <c r="BV15" s="29" t="n"/>
-      <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="30" t="n"/>
-      <c r="BY15" s="27" t="n"/>
-      <c r="BZ15" s="24" t="n"/>
-      <c r="CA15" s="31" t="n"/>
-      <c r="CB15" s="24" t="n"/>
-      <c r="CC15" s="24" t="n"/>
-      <c r="CD15" s="24" t="n"/>
-      <c r="CE15" s="24" t="n"/>
-      <c r="CF15" s="24" t="n"/>
-      <c r="CG15" s="24" t="n"/>
-      <c r="CH15" s="24" t="n"/>
-      <c r="CI15" s="24" t="n"/>
-      <c r="CJ15" s="24" t="n"/>
-      <c r="CK15" s="24" t="n"/>
-      <c r="CL15" s="24" t="n"/>
-      <c r="CM15" s="24" t="n"/>
-      <c r="CN15" s="24" t="n"/>
-      <c r="CO15" s="24" t="n"/>
-      <c r="CP15" s="24" t="n"/>
-      <c r="CQ15" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>db1dc943d75f40cf</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T18:08:55.998248Z</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T10:30:00Z</t>
-        </is>
-      </c>
-      <c r="D16" s="24" t="inlineStr">
-        <is>
-          <t>67514</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="G16" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="H16" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I16" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J16" s="25" t="n"/>
-      <c r="K16" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L16" s="26" t="n">
-        <v>-163</v>
-      </c>
-      <c r="M16" s="27" t="n">
-        <v>1.613497</v>
-      </c>
-      <c r="N16" s="28" t="n">
-        <v>0.619772</v>
-      </c>
-      <c r="O16" s="28" t="n">
-        <v>0.639896</v>
-      </c>
-      <c r="P16" s="28" t="n"/>
-      <c r="Q16" s="28" t="n">
-        <v>0.020124</v>
-      </c>
-      <c r="R16" s="26" t="n">
-        <v>30</v>
-      </c>
-      <c r="S16" s="29" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="T16" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U16" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V16" s="24" t="n"/>
-      <c r="W16" s="26" t="n"/>
-      <c r="X16" s="26" t="n"/>
-      <c r="Y16" s="25" t="n"/>
-      <c r="Z16" s="26" t="n"/>
-      <c r="AA16" s="28" t="n"/>
-      <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="30" t="n"/>
-      <c r="AD16" s="24" t="n"/>
-      <c r="AE16" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-cs2-era-psna-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF16" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG16" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH16" s="24" t="n"/>
-      <c r="AI16" s="31" t="n"/>
-      <c r="AJ16" s="31" t="n"/>
-      <c r="AK16" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL16" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM16" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN16" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO16" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP16" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="AQ16" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="AR16" s="24" t="inlineStr">
-        <is>
-          <t>Passion Academy</t>
-        </is>
-      </c>
-      <c r="AS16" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="AT16" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="AU16" s="24" t="inlineStr">
-        <is>
-          <t>EAC Rising</t>
-        </is>
-      </c>
-      <c r="AV16" s="24" t="n"/>
-      <c r="AW16" s="24" t="n"/>
-      <c r="AX16" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY16" s="24" t="n"/>
-      <c r="AZ16" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA16" s="24" t="inlineStr">
-        <is>
-          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
-        </is>
-      </c>
-      <c r="BB16" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC16" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD16" s="24" t="inlineStr">
-        <is>
-          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
-        </is>
-      </c>
-      <c r="BE16" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF16" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG16" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH16" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T18:08:48.789246Z</t>
-        </is>
-      </c>
-      <c r="BI16" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ16" s="25" t="n"/>
-      <c r="BK16" s="26" t="n">
-        <v>-163</v>
-      </c>
-      <c r="BL16" s="27" t="n">
-        <v>1.613497</v>
-      </c>
-      <c r="BM16" s="28" t="n">
-        <v>0.619772</v>
-      </c>
-      <c r="BN16" s="28" t="n"/>
-      <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="25" t="n"/>
-      <c r="BQ16" s="27" t="n"/>
-      <c r="BR16" s="28" t="n"/>
-      <c r="BS16" s="28" t="n"/>
-      <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="25" t="n"/>
-      <c r="BV16" s="29" t="n"/>
-      <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="30" t="n"/>
-      <c r="BY16" s="27" t="n"/>
-      <c r="BZ16" s="24" t="n"/>
-      <c r="CA16" s="31" t="n"/>
-      <c r="CB16" s="24" t="n"/>
-      <c r="CC16" s="24" t="n"/>
-      <c r="CD16" s="24" t="n"/>
-      <c r="CE16" s="24" t="n"/>
-      <c r="CF16" s="24" t="n"/>
-      <c r="CG16" s="24" t="n"/>
-      <c r="CH16" s="24" t="n"/>
-      <c r="CI16" s="24" t="n"/>
-      <c r="CJ16" s="24" t="n"/>
-      <c r="CK16" s="24" t="n"/>
-      <c r="CL16" s="24" t="n"/>
-      <c r="CM16" s="24" t="n"/>
-      <c r="CN16" s="24" t="n"/>
-      <c r="CO16" s="24" t="n"/>
-      <c r="CP16" s="24" t="n"/>
-      <c r="CQ16" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>d60a6e820d4f4adc</t>
-        </is>
-      </c>
-      <c r="B17" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T18:08:55.998248Z</t>
-        </is>
-      </c>
-      <c r="C17" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T14:00:00Z</t>
-        </is>
-      </c>
-      <c r="D17" s="24" t="inlineStr">
-        <is>
-          <t>69268</t>
-        </is>
-      </c>
-      <c r="E17" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F17" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="G17" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="H17" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I17" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J17" s="25" t="n"/>
-      <c r="K17" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L17" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="M17" s="27" t="n">
-        <v>1.561798</v>
-      </c>
-      <c r="N17" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="O17" s="28" t="n">
-        <v>0.663041</v>
-      </c>
-      <c r="P17" s="28" t="n"/>
-      <c r="Q17" s="28" t="n">
-        <v>0.022753</v>
-      </c>
-      <c r="R17" s="26" t="n">
-        <v>31</v>
-      </c>
-      <c r="S17" s="29" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="T17" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U17" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V17" s="24" t="n"/>
-      <c r="W17" s="26" t="n"/>
-      <c r="X17" s="26" t="n"/>
-      <c r="Y17" s="25" t="n"/>
-      <c r="Z17" s="26" t="n"/>
-      <c r="AA17" s="28" t="n"/>
-      <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="30" t="n"/>
-      <c r="AD17" s="24" t="n"/>
-      <c r="AE17" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF17" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG17" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH17" s="24" t="n"/>
-      <c r="AI17" s="31" t="n"/>
-      <c r="AJ17" s="31" t="n"/>
-      <c r="AK17" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL17" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM17" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN17" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO17" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP17" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="AQ17" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="AR17" s="24" t="inlineStr">
-        <is>
-          <t>ex-Young Ninjas</t>
-        </is>
-      </c>
-      <c r="AS17" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="AT17" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="AU17" s="24" t="inlineStr">
-        <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="AV17" s="24" t="n"/>
-      <c r="AW17" s="24" t="n"/>
-      <c r="AX17" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY17" s="24" t="n"/>
-      <c r="AZ17" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA17" s="24" t="inlineStr">
-        <is>
-          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
-        </is>
-      </c>
-      <c r="BB17" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC17" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD17" s="24" t="inlineStr">
-        <is>
-          <t>d5fa90971ced522e0070399e9eeaba0b323d1e6ef1030b6470d86e8cb482d801</t>
-        </is>
-      </c>
-      <c r="BE17" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF17" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG17" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH17" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T18:08:51.418739Z</t>
-        </is>
-      </c>
-      <c r="BI17" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ17" s="25" t="n"/>
-      <c r="BK17" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="BL17" s="27" t="n">
-        <v>1.561798</v>
-      </c>
-      <c r="BM17" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="BN17" s="28" t="n"/>
-      <c r="BO17" s="28" t="n"/>
-      <c r="BP17" s="25" t="n"/>
-      <c r="BQ17" s="27" t="n"/>
-      <c r="BR17" s="28" t="n"/>
-      <c r="BS17" s="28" t="n"/>
-      <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="25" t="n"/>
-      <c r="BV17" s="29" t="n"/>
-      <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="30" t="n"/>
-      <c r="BY17" s="27" t="n"/>
-      <c r="BZ17" s="24" t="n"/>
-      <c r="CA17" s="31" t="n"/>
-      <c r="CB17" s="24" t="n"/>
-      <c r="CC17" s="24" t="n"/>
-      <c r="CD17" s="24" t="n"/>
-      <c r="CE17" s="24" t="n"/>
-      <c r="CF17" s="24" t="n"/>
-      <c r="CG17" s="24" t="n"/>
-      <c r="CH17" s="24" t="n"/>
-      <c r="CI17" s="24" t="n"/>
-      <c r="CJ17" s="24" t="n"/>
-      <c r="CK17" s="24" t="n"/>
-      <c r="CL17" s="24" t="n"/>
-      <c r="CM17" s="24" t="n"/>
-      <c r="CN17" s="24" t="n"/>
-      <c r="CO17" s="24" t="n"/>
-      <c r="CP17" s="24" t="n"/>
-      <c r="CQ17" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix: redact Odds API key from errors, mark stale P1 claims in MASTER.md, 654 tests pass
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ14" headerRowCount="1">
-  <autoFilter ref="A1:CQ14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ17" headerRowCount="1">
+  <autoFilter ref="A1:CQ17"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$14)</f>
+        <f>COUNTA('Picks'!$A$2:$A$17)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$17,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$17,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")/(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$17)/SUM('Picks'!$BX$2:$BX$17),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$14)</f>
+        <f>SUM('Picks'!$BY$2:$BY$17)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$17,"&lt;&gt;",'Picks'!$AB$2:$AB$17),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$17,'Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ14"/>
+  <dimension ref="A1:CQ17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5266,6 +5266,807 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>95d87d5169fc4ae9</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:24:44.992034Z</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T10:00:00Z</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>68289</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J15" s="25" t="n"/>
+      <c r="K15" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L15" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M15" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N15" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O15" s="28" t="n">
+        <v>0.599274</v>
+      </c>
+      <c r="P15" s="28" t="n"/>
+      <c r="Q15" s="28" t="n">
+        <v>0.019442</v>
+      </c>
+      <c r="R15" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="S15" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U15" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="n"/>
+      <c r="W15" s="26" t="n"/>
+      <c r="X15" s="26" t="n"/>
+      <c r="Y15" s="25" t="n"/>
+      <c r="Z15" s="26" t="n"/>
+      <c r="AA15" s="28" t="n"/>
+      <c r="AB15" s="28" t="n"/>
+      <c r="AC15" s="30" t="n"/>
+      <c r="AD15" s="24" t="n"/>
+      <c r="AE15" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF15" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG15" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH15" s="24" t="n"/>
+      <c r="AI15" s="31" t="n"/>
+      <c r="AJ15" s="31" t="n"/>
+      <c r="AK15" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL15" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM15" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN15" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO15" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AQ15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AR15" s="24" t="inlineStr">
+        <is>
+          <t>FURY</t>
+        </is>
+      </c>
+      <c r="AS15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AT15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AU15" s="24" t="inlineStr">
+        <is>
+          <t>Mindfreak</t>
+        </is>
+      </c>
+      <c r="AV15" s="24" t="n"/>
+      <c r="AW15" s="24" t="n"/>
+      <c r="AX15" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY15" s="24" t="n"/>
+      <c r="AZ15" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA15" s="24" t="inlineStr">
+        <is>
+          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+        </is>
+      </c>
+      <c r="BB15" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD15" s="24" t="inlineStr">
+        <is>
+          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+        </is>
+      </c>
+      <c r="BE15" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF15" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG15" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:24:35.118991Z</t>
+        </is>
+      </c>
+      <c r="BI15" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ15" s="25" t="n"/>
+      <c r="BK15" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL15" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM15" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN15" s="28" t="n"/>
+      <c r="BO15" s="28" t="n"/>
+      <c r="BP15" s="25" t="n"/>
+      <c r="BQ15" s="27" t="n"/>
+      <c r="BR15" s="28" t="n"/>
+      <c r="BS15" s="28" t="n"/>
+      <c r="BT15" s="28" t="n"/>
+      <c r="BU15" s="25" t="n"/>
+      <c r="BV15" s="29" t="n"/>
+      <c r="BW15" s="24" t="n"/>
+      <c r="BX15" s="30" t="n"/>
+      <c r="BY15" s="27" t="n"/>
+      <c r="BZ15" s="24" t="n"/>
+      <c r="CA15" s="31" t="n"/>
+      <c r="CB15" s="24" t="n"/>
+      <c r="CC15" s="24" t="n"/>
+      <c r="CD15" s="24" t="n"/>
+      <c r="CE15" s="24" t="n"/>
+      <c r="CF15" s="24" t="n"/>
+      <c r="CG15" s="24" t="n"/>
+      <c r="CH15" s="24" t="n"/>
+      <c r="CI15" s="24" t="n"/>
+      <c r="CJ15" s="24" t="n"/>
+      <c r="CK15" s="24" t="n"/>
+      <c r="CL15" s="24" t="n"/>
+      <c r="CM15" s="24" t="n"/>
+      <c r="CN15" s="24" t="n"/>
+      <c r="CO15" s="24" t="n"/>
+      <c r="CP15" s="24" t="n"/>
+      <c r="CQ15" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>252f5baff6014e4d</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:24:44.992034Z</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T10:30:00Z</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>67514</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Passion Academy</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>EAC Rising</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="M16" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="N16" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="O16" s="28" t="n">
+        <v>0.640004</v>
+      </c>
+      <c r="P16" s="28" t="n"/>
+      <c r="Q16" s="28" t="n">
+        <v>0.020232</v>
+      </c>
+      <c r="R16" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="S16" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U16" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V16" s="24" t="n"/>
+      <c r="W16" s="26" t="n"/>
+      <c r="X16" s="26" t="n"/>
+      <c r="Y16" s="25" t="n"/>
+      <c r="Z16" s="26" t="n"/>
+      <c r="AA16" s="28" t="n"/>
+      <c r="AB16" s="28" t="n"/>
+      <c r="AC16" s="30" t="n"/>
+      <c r="AD16" s="24" t="n"/>
+      <c r="AE16" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-cs2-era-psna-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF16" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG16" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH16" s="24" t="n"/>
+      <c r="AI16" s="31" t="n"/>
+      <c r="AJ16" s="31" t="n"/>
+      <c r="AK16" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL16" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN16" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO16" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP16" s="24" t="inlineStr">
+        <is>
+          <t>Passion Academy</t>
+        </is>
+      </c>
+      <c r="AQ16" s="24" t="inlineStr">
+        <is>
+          <t>Passion Academy</t>
+        </is>
+      </c>
+      <c r="AR16" s="24" t="inlineStr">
+        <is>
+          <t>Passion Academy</t>
+        </is>
+      </c>
+      <c r="AS16" s="24" t="inlineStr">
+        <is>
+          <t>EAC Rising</t>
+        </is>
+      </c>
+      <c r="AT16" s="24" t="inlineStr">
+        <is>
+          <t>EAC Rising</t>
+        </is>
+      </c>
+      <c r="AU16" s="24" t="inlineStr">
+        <is>
+          <t>EAC Rising</t>
+        </is>
+      </c>
+      <c r="AV16" s="24" t="n"/>
+      <c r="AW16" s="24" t="n"/>
+      <c r="AX16" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY16" s="24" t="n"/>
+      <c r="AZ16" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA16" s="24" t="inlineStr">
+        <is>
+          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+        </is>
+      </c>
+      <c r="BB16" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD16" s="24" t="inlineStr">
+        <is>
+          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+        </is>
+      </c>
+      <c r="BE16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF16" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG16" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH16" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:24:37.624827Z</t>
+        </is>
+      </c>
+      <c r="BI16" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ16" s="25" t="n"/>
+      <c r="BK16" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="BL16" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="BM16" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="BN16" s="28" t="n"/>
+      <c r="BO16" s="28" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
+      <c r="BR16" s="28" t="n"/>
+      <c r="BS16" s="28" t="n"/>
+      <c r="BT16" s="28" t="n"/>
+      <c r="BU16" s="25" t="n"/>
+      <c r="BV16" s="29" t="n"/>
+      <c r="BW16" s="24" t="n"/>
+      <c r="BX16" s="30" t="n"/>
+      <c r="BY16" s="27" t="n"/>
+      <c r="BZ16" s="24" t="n"/>
+      <c r="CA16" s="31" t="n"/>
+      <c r="CB16" s="24" t="n"/>
+      <c r="CC16" s="24" t="n"/>
+      <c r="CD16" s="24" t="n"/>
+      <c r="CE16" s="24" t="n"/>
+      <c r="CF16" s="24" t="n"/>
+      <c r="CG16" s="24" t="n"/>
+      <c r="CH16" s="24" t="n"/>
+      <c r="CI16" s="24" t="n"/>
+      <c r="CJ16" s="24" t="n"/>
+      <c r="CK16" s="24" t="n"/>
+      <c r="CL16" s="24" t="n"/>
+      <c r="CM16" s="24" t="n"/>
+      <c r="CN16" s="24" t="n"/>
+      <c r="CO16" s="24" t="n"/>
+      <c r="CP16" s="24" t="n"/>
+      <c r="CQ16" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>2965fad2679e43bb</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:24:44.992034Z</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>69268</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J17" s="25" t="n"/>
+      <c r="K17" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M17" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N17" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O17" s="28" t="n">
+        <v>0.663166</v>
+      </c>
+      <c r="P17" s="28" t="n"/>
+      <c r="Q17" s="28" t="n">
+        <v>0.022878</v>
+      </c>
+      <c r="R17" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="S17" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T17" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U17" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V17" s="24" t="n"/>
+      <c r="W17" s="26" t="n"/>
+      <c r="X17" s="26" t="n"/>
+      <c r="Y17" s="25" t="n"/>
+      <c r="Z17" s="26" t="n"/>
+      <c r="AA17" s="28" t="n"/>
+      <c r="AB17" s="28" t="n"/>
+      <c r="AC17" s="30" t="n"/>
+      <c r="AD17" s="24" t="n"/>
+      <c r="AE17" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+        </is>
+      </c>
+      <c r="AF17" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG17" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH17" s="24" t="n"/>
+      <c r="AI17" s="31" t="n"/>
+      <c r="AJ17" s="31" t="n"/>
+      <c r="AK17" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL17" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM17" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN17" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO17" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AQ17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AR17" s="24" t="inlineStr">
+        <is>
+          <t>ex-Young Ninjas</t>
+        </is>
+      </c>
+      <c r="AS17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AT17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AU17" s="24" t="inlineStr">
+        <is>
+          <t>SPARTA</t>
+        </is>
+      </c>
+      <c r="AV17" s="24" t="n"/>
+      <c r="AW17" s="24" t="n"/>
+      <c r="AX17" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY17" s="24" t="n"/>
+      <c r="AZ17" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA17" s="24" t="inlineStr">
+        <is>
+          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+        </is>
+      </c>
+      <c r="BB17" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC17" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD17" s="24" t="inlineStr">
+        <is>
+          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+        </is>
+      </c>
+      <c r="BE17" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF17" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG17" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH17" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-02T18:24:40.237935Z</t>
+        </is>
+      </c>
+      <c r="BI17" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ17" s="25" t="n"/>
+      <c r="BK17" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL17" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM17" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN17" s="28" t="n"/>
+      <c r="BO17" s="28" t="n"/>
+      <c r="BP17" s="25" t="n"/>
+      <c r="BQ17" s="27" t="n"/>
+      <c r="BR17" s="28" t="n"/>
+      <c r="BS17" s="28" t="n"/>
+      <c r="BT17" s="28" t="n"/>
+      <c r="BU17" s="25" t="n"/>
+      <c r="BV17" s="29" t="n"/>
+      <c r="BW17" s="24" t="n"/>
+      <c r="BX17" s="30" t="n"/>
+      <c r="BY17" s="27" t="n"/>
+      <c r="BZ17" s="24" t="n"/>
+      <c r="CA17" s="31" t="n"/>
+      <c r="CB17" s="24" t="n"/>
+      <c r="CC17" s="24" t="n"/>
+      <c r="CD17" s="24" t="n"/>
+      <c r="CE17" s="24" t="n"/>
+      <c r="CF17" s="24" t="n"/>
+      <c r="CG17" s="24" t="n"/>
+      <c r="CH17" s="24" t="n"/>
+      <c r="CI17" s="24" t="n"/>
+      <c r="CJ17" s="24" t="n"/>
+      <c r="CK17" s="24" t="n"/>
+      <c r="CL17" s="24" t="n"/>
+      <c r="CM17" s="24" t="n"/>
+      <c r="CN17" s="24" t="n"/>
+      <c r="CO17" s="24" t="n"/>
+      <c r="CP17" s="24" t="n"/>
+      <c r="CQ17" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
chore: per-sport Main/Flat ledger migration + production data sync
Commits the data side of the per-sport ledger split (code landed in
95b6c92): data/main/{mlb,wnba,soccer,tennis}.xlsx and data/flat/{same}.xlsx
replace the old shared data/picks.xlsx and data/flat_picks.xlsx, which are
now deleted. This was already run against production and verified end to
end in the prior session but never staged.

Also syncs everything the daily cron wrote across today's several runs
(settlements, new picks, esports/international-baseball history refresh,
odds snapshots, model ledgers) plus the pre-migration reconciliation
backups (backups/) taken before this split and before the earlier gate
reconciliation.

verify-chain: chain_intact, zero breaks. Zero duplicates across all 26
Main/Flat/Research/Gated ledger files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gated_research/cs2.xlsx
+++ b/data/gated_research/cs2.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ17" headerRowCount="1">
-  <autoFilter ref="A1:CQ17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ21" headerRowCount="1">
+  <autoFilter ref="A1:CQ21"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$17)</f>
+        <f>COUNTA('Picks'!$A$2:$A$21)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$17,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$21,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")+COUNTIFS('Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$17,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$21,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")/(COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"win")+COUNTIFS('Picks'!$BX$2:$BX$17,"&gt;0",'Picks'!$V$2:$V$17,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"win")/(COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"win")+COUNTIFS('Picks'!$BX$2:$BX$21,"&gt;0",'Picks'!$V$2:$V$21,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$17)/SUM('Picks'!$BX$2:$BX$17),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$21)/SUM('Picks'!$BX$2:$BX$21),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$17)</f>
+        <f>SUM('Picks'!$BY$2:$BY$21)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$17,"&lt;&gt;",'Picks'!$AB$2:$AB$17),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$21,"&lt;&gt;",'Picks'!$AB$2:$AB$21),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$21,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$17,'Picks'!$AM$2:$AM$17,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$21,'Picks'!$AM$2:$AM$21,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$21,'Picks'!$H$2:$H$21,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A14,'Picks'!$U$2:$U$17,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$21,'Picks'!$H$2:$H$21,$A14,'Picks'!$U$2:$U$21,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$21,'Picks'!$H$2:$H$21,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A15,'Picks'!$U$2:$U$17,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$21,'Picks'!$H$2:$H$21,$A15,'Picks'!$U$2:$U$21,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled",'Picks'!$V$2:$V$17,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled",'Picks'!$V$2:$V$21,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$17,'Picks'!$H$2:$H$17,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$21,'Picks'!$H$2:$H$21,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$17,'Picks'!$H$2:$H$17,$A16,'Picks'!$U$2:$U$17,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$21,'Picks'!$H$2:$H$21,$A16,'Picks'!$U$2:$U$21,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ17"/>
+  <dimension ref="A1:CQ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4817,18 +4817,28 @@
       </c>
       <c r="U13" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V13" s="24" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V13" s="24" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
       <c r="W13" s="26" t="n"/>
       <c r="X13" s="26" t="n"/>
       <c r="Y13" s="25" t="n"/>
       <c r="Z13" s="26" t="n"/>
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="30" t="n"/>
-      <c r="AD13" s="24" t="n"/>
+      <c r="AC13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T02:34:48.118824Z</t>
+        </is>
+      </c>
       <c r="AE13" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.5300 (market_slug=aec-cs2-dc-for-2026-08-02).</t>
@@ -4977,7 +4987,11 @@
       <c r="BT13" s="28" t="n"/>
       <c r="BU13" s="25" t="n"/>
       <c r="BV13" s="29" t="n"/>
-      <c r="BW13" s="24" t="n"/>
+      <c r="BW13" s="24" t="inlineStr">
+        <is>
+          <t>esports market settled to a non-binary price (forfeit/postponement per market rules)</t>
+        </is>
+      </c>
       <c r="BX13" s="30" t="n"/>
       <c r="BY13" s="27" t="n"/>
       <c r="BZ13" s="24" t="n"/>
@@ -5080,18 +5094,28 @@
       </c>
       <c r="U14" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V14" s="24" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V14" s="24" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
       <c r="W14" s="26" t="n"/>
       <c r="X14" s="26" t="n"/>
       <c r="Y14" s="25" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="30" t="n"/>
-      <c r="AD14" s="24" t="n"/>
+      <c r="AC14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T02:34:49.249923Z</t>
+        </is>
+      </c>
       <c r="AE14" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.6600 (market_slug=aec-cs2-mta-enjoy-2026-08-02).</t>
@@ -5240,7 +5264,11 @@
       <c r="BT14" s="28" t="n"/>
       <c r="BU14" s="25" t="n"/>
       <c r="BV14" s="29" t="n"/>
-      <c r="BW14" s="24" t="n"/>
+      <c r="BW14" s="24" t="inlineStr">
+        <is>
+          <t>esports market settled to a non-binary price (forfeit/postponement per market rules)</t>
+        </is>
+      </c>
       <c r="BX14" s="30" t="n"/>
       <c r="BY14" s="27" t="n"/>
       <c r="BZ14" s="24" t="n"/>
@@ -5269,22 +5297,22 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>95d87d5169fc4ae9</t>
+          <t>3e5ca2341bea45d1</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T18:24:44.992034Z</t>
+          <t>2026-08-03T10:14:59.378487Z</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-03T10:00:00Z</t>
+          <t>2026-08-03T10:30:00Z</t>
         </is>
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>68289</t>
+          <t>67514</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
@@ -5294,12 +5322,12 @@
       </c>
       <c r="F15" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="G15" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="H15" s="24" t="inlineStr">
@@ -5319,26 +5347,26 @@
         </is>
       </c>
       <c r="L15" s="26" t="n">
-        <v>-138</v>
+        <v>-156</v>
       </c>
       <c r="M15" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.641026</v>
       </c>
       <c r="N15" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.609375</v>
       </c>
       <c r="O15" s="28" t="n">
-        <v>0.599274</v>
+        <v>0.639821</v>
       </c>
       <c r="P15" s="28" t="n"/>
       <c r="Q15" s="28" t="n">
-        <v>0.019442</v>
+        <v>0.030446</v>
       </c>
       <c r="R15" s="26" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="S15" s="29" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="T15" s="24" t="inlineStr">
         <is>
@@ -5347,21 +5375,41 @@
       </c>
       <c r="U15" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V15" s="24" t="n"/>
-      <c r="W15" s="26" t="n"/>
-      <c r="X15" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W15" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y15" s="25" t="n"/>
-      <c r="Z15" s="26" t="n"/>
-      <c r="AA15" s="28" t="n"/>
-      <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n"/>
-      <c r="AD15" s="24" t="n"/>
+      <c r="Z15" s="26" t="n">
+        <v>-156</v>
+      </c>
+      <c r="AA15" s="28" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="AB15" s="28" t="n">
+        <v>0.000625</v>
+      </c>
+      <c r="AC15" s="30" t="n">
+        <v>0.9615</v>
+      </c>
+      <c r="AD15" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-03T13:27:35.671440Z</t>
+        </is>
+      </c>
       <c r="AE15" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-mf-fury-2026-08-03).</t>
+          <t>Neutral Elo baseline; executable ask 0.6100 (market_slug=aec-cs2-era-psna-2026-08-03).</t>
         </is>
       </c>
       <c r="AF15" s="31" t="inlineStr">
@@ -5402,32 +5450,32 @@
       </c>
       <c r="AP15" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="AQ15" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="AR15" s="24" t="inlineStr">
         <is>
-          <t>FURY</t>
+          <t>Passion Academy</t>
         </is>
       </c>
       <c r="AS15" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="AT15" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="AU15" s="24" t="inlineStr">
         <is>
-          <t>Mindfreak</t>
+          <t>EAC Rising</t>
         </is>
       </c>
       <c r="AV15" s="24" t="n"/>
@@ -5445,7 +5493,7 @@
       </c>
       <c r="BA15" s="24" t="inlineStr">
         <is>
-          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+          <t>a67b482e0cc299818c9d6a6183162092d6b3cbeea4f974054606da1c44c3bd99</t>
         </is>
       </c>
       <c r="BB15" s="24" t="inlineStr">
@@ -5460,7 +5508,7 @@
       </c>
       <c r="BD15" s="24" t="inlineStr">
         <is>
-          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+          <t>a67b482e0cc299818c9d6a6183162092d6b3cbeea4f974054606da1c44c3bd99</t>
         </is>
       </c>
       <c r="BE15" s="24" t="inlineStr">
@@ -5480,7 +5528,7 @@
       </c>
       <c r="BH15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T18:24:35.118991Z</t>
+          <t>2026-08-03T10:14:38.370048Z</t>
         </is>
       </c>
       <c r="BI15" s="24" t="inlineStr">
@@ -5490,19 +5538,23 @@
       </c>
       <c r="BJ15" s="25" t="n"/>
       <c r="BK15" s="26" t="n">
-        <v>-138</v>
+        <v>-156</v>
       </c>
       <c r="BL15" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.641026</v>
       </c>
       <c r="BM15" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.609375</v>
       </c>
       <c r="BN15" s="28" t="n"/>
       <c r="BO15" s="28" t="n"/>
       <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
-      <c r="BR15" s="28" t="n"/>
+      <c r="BQ15" s="27" t="n">
+        <v>1.641026</v>
+      </c>
+      <c r="BR15" s="28" t="n">
+        <v>0.61</v>
+      </c>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
       <c r="BU15" s="25" t="n"/>
@@ -5536,22 +5588,22 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>252f5baff6014e4d</t>
+          <t>02ebc095ca494cd9</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T18:24:44.992034Z</t>
+          <t>2026-08-03T19:54:57.645683Z</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-03T10:30:00Z</t>
+          <t>2026-08-03T21:00:00Z</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>67514</t>
+          <t>70532</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
@@ -5561,12 +5613,12 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>Passion Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
-          <t>EAC Rising</t>
+          <t>ODDIK</t>
         </is>
       </c>
       <c r="H16" s="24" t="inlineStr">
@@ -5586,23 +5638,23 @@
         </is>
       </c>
       <c r="L16" s="26" t="n">
-        <v>-163</v>
+        <v>-150</v>
       </c>
       <c r="M16" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.666667</v>
       </c>
       <c r="N16" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.6</v>
       </c>
       <c r="O16" s="28" t="n">
-        <v>0.640004</v>
+        <v>0.6304380000000001</v>
       </c>
       <c r="P16" s="28" t="n"/>
       <c r="Q16" s="28" t="n">
-        <v>0.020232</v>
+        <v>0.030438</v>
       </c>
       <c r="R16" s="26" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="S16" s="29" t="n">
         <v>1.5</v>
@@ -5628,7 +5680,7 @@
       <c r="AD16" s="24" t="n"/>
       <c r="AE16" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-cs2-era-psna-2026-08-03).</t>
+          <t>Neutral Elo baseline; executable ask 0.6000 (market_slug=aec-cs2-odk-reda-2026-08-03).</t>
         </is>
       </c>
       <c r="AF16" s="31" t="inlineStr">
@@ -5669,32 +5721,32 @@
       </c>
       <c r="AP16" s="24" t="inlineStr">
         <is>
-          <t>Passion Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="AQ16" s="24" t="inlineStr">
         <is>
-          <t>Passion Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="AR16" s="24" t="inlineStr">
         <is>
-          <t>Passion Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="AS16" s="24" t="inlineStr">
         <is>
-          <t>EAC Rising</t>
+          <t>ODDIK</t>
         </is>
       </c>
       <c r="AT16" s="24" t="inlineStr">
         <is>
-          <t>EAC Rising</t>
+          <t>ODDIK</t>
         </is>
       </c>
       <c r="AU16" s="24" t="inlineStr">
         <is>
-          <t>EAC Rising</t>
+          <t>ODDIK</t>
         </is>
       </c>
       <c r="AV16" s="24" t="n"/>
@@ -5712,7 +5764,7 @@
       </c>
       <c r="BA16" s="24" t="inlineStr">
         <is>
-          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+          <t>49e72bc47e8b746259057b18a0727b3402ae02f53069edfae5b6532757438c2c</t>
         </is>
       </c>
       <c r="BB16" s="24" t="inlineStr">
@@ -5727,7 +5779,7 @@
       </c>
       <c r="BD16" s="24" t="inlineStr">
         <is>
-          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+          <t>49e72bc47e8b746259057b18a0727b3402ae02f53069edfae5b6532757438c2c</t>
         </is>
       </c>
       <c r="BE16" s="24" t="inlineStr">
@@ -5747,7 +5799,7 @@
       </c>
       <c r="BH16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T18:24:37.624827Z</t>
+          <t>2026-08-03T19:54:46.268393Z</t>
         </is>
       </c>
       <c r="BI16" s="24" t="inlineStr">
@@ -5757,13 +5809,13 @@
       </c>
       <c r="BJ16" s="25" t="n"/>
       <c r="BK16" s="26" t="n">
-        <v>-163</v>
+        <v>-150</v>
       </c>
       <c r="BL16" s="27" t="n">
-        <v>1.613497</v>
+        <v>1.666667</v>
       </c>
       <c r="BM16" s="28" t="n">
-        <v>0.619772</v>
+        <v>0.6</v>
       </c>
       <c r="BN16" s="28" t="n"/>
       <c r="BO16" s="28" t="n"/>
@@ -5803,22 +5855,22 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>2965fad2679e43bb</t>
+          <t>35497da3e6964fbc</t>
         </is>
       </c>
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T18:24:44.992034Z</t>
+          <t>2026-08-04T02:01:00.694416Z</t>
         </is>
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>2026-08-03T14:00:00Z</t>
+          <t>2026-08-04T11:00:00Z</t>
         </is>
       </c>
       <c r="D17" s="24" t="inlineStr">
         <is>
-          <t>69268</t>
+          <t>68302</t>
         </is>
       </c>
       <c r="E17" s="24" t="inlineStr">
@@ -5828,12 +5880,12 @@
       </c>
       <c r="F17" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="G17" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Sashi Esport</t>
         </is>
       </c>
       <c r="H17" s="24" t="inlineStr">
@@ -5853,26 +5905,26 @@
         </is>
       </c>
       <c r="L17" s="26" t="n">
-        <v>-178</v>
+        <v>117</v>
       </c>
       <c r="M17" s="27" t="n">
-        <v>1.561798</v>
+        <v>2.17</v>
       </c>
       <c r="N17" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.460829</v>
       </c>
       <c r="O17" s="28" t="n">
-        <v>0.663166</v>
+        <v>0.551006</v>
       </c>
       <c r="P17" s="28" t="n"/>
       <c r="Q17" s="28" t="n">
-        <v>0.022878</v>
+        <v>0.09017699999999999</v>
       </c>
       <c r="R17" s="26" t="n">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="S17" s="29" t="n">
-        <v>1.75</v>
+        <v>1</v>
       </c>
       <c r="T17" s="24" t="inlineStr">
         <is>
@@ -5895,7 +5947,7 @@
       <c r="AD17" s="24" t="n"/>
       <c r="AE17" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.6400 (market_slug=aec-cs2-sparta-eyn-2026-08-03).</t>
+          <t>Neutral Elo baseline; executable ask 0.4600 (market_slug=aec-cs2-sashi-pha-2026-08-04).</t>
         </is>
       </c>
       <c r="AF17" s="31" t="inlineStr">
@@ -5936,32 +5988,32 @@
       </c>
       <c r="AP17" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="AQ17" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="AR17" s="24" t="inlineStr">
         <is>
-          <t>ex-Young Ninjas</t>
+          <t>Phantom</t>
         </is>
       </c>
       <c r="AS17" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Sashi Esport</t>
         </is>
       </c>
       <c r="AT17" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Sashi Esport</t>
         </is>
       </c>
       <c r="AU17" s="24" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>Sashi Esport</t>
         </is>
       </c>
       <c r="AV17" s="24" t="n"/>
@@ -5979,7 +6031,7 @@
       </c>
       <c r="BA17" s="24" t="inlineStr">
         <is>
-          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
         </is>
       </c>
       <c r="BB17" s="24" t="inlineStr">
@@ -5994,7 +6046,7 @@
       </c>
       <c r="BD17" s="24" t="inlineStr">
         <is>
-          <t>0393e290b17b4d34bf783a8173fb53c53aebc8558545e4c0778b6e017fd0a405</t>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
         </is>
       </c>
       <c r="BE17" s="24" t="inlineStr">
@@ -6014,7 +6066,7 @@
       </c>
       <c r="BH17" s="24" t="inlineStr">
         <is>
-          <t>2026-08-02T18:24:40.237935Z</t>
+          <t>2026-08-04T02:00:44.822978Z</t>
         </is>
       </c>
       <c r="BI17" s="24" t="inlineStr">
@@ -6024,13 +6076,13 @@
       </c>
       <c r="BJ17" s="25" t="n"/>
       <c r="BK17" s="26" t="n">
-        <v>-178</v>
+        <v>117</v>
       </c>
       <c r="BL17" s="27" t="n">
-        <v>1.561798</v>
+        <v>2.17</v>
       </c>
       <c r="BM17" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.460829</v>
       </c>
       <c r="BN17" s="28" t="n"/>
       <c r="BO17" s="28" t="n"/>
@@ -6067,6 +6119,1074 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>5917a6df4bb84597</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T02:01:00.694416Z</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T11:00:00Z</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>71501</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>Betclic Apogee Esports</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
+        <is>
+          <t>Acend</t>
+        </is>
+      </c>
+      <c r="H18" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I18" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J18" s="25" t="n"/>
+      <c r="K18" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M18" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N18" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O18" s="28" t="n">
+        <v>0.691599</v>
+      </c>
+      <c r="P18" s="28" t="n"/>
+      <c r="Q18" s="28" t="n">
+        <v>0.111767</v>
+      </c>
+      <c r="R18" s="26" t="n">
+        <v>76</v>
+      </c>
+      <c r="S18" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T18" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U18" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V18" s="24" t="n"/>
+      <c r="W18" s="26" t="n"/>
+      <c r="X18" s="26" t="n"/>
+      <c r="Y18" s="25" t="n"/>
+      <c r="Z18" s="26" t="n"/>
+      <c r="AA18" s="28" t="n"/>
+      <c r="AB18" s="28" t="n"/>
+      <c r="AC18" s="30" t="n"/>
+      <c r="AD18" s="24" t="n"/>
+      <c r="AE18" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5800 (market_slug=aec-cs2-ace-bca-2026-08-04).</t>
+        </is>
+      </c>
+      <c r="AF18" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG18" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH18" s="24" t="n"/>
+      <c r="AI18" s="31" t="n"/>
+      <c r="AJ18" s="31" t="n"/>
+      <c r="AK18" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL18" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM18" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN18" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO18" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP18" s="24" t="inlineStr">
+        <is>
+          <t>Betclic Apogee Esports</t>
+        </is>
+      </c>
+      <c r="AQ18" s="24" t="inlineStr">
+        <is>
+          <t>Betclic Apogee Esports</t>
+        </is>
+      </c>
+      <c r="AR18" s="24" t="inlineStr">
+        <is>
+          <t>Betclic Apogee Esports</t>
+        </is>
+      </c>
+      <c r="AS18" s="24" t="inlineStr">
+        <is>
+          <t>Acend</t>
+        </is>
+      </c>
+      <c r="AT18" s="24" t="inlineStr">
+        <is>
+          <t>Acend</t>
+        </is>
+      </c>
+      <c r="AU18" s="24" t="inlineStr">
+        <is>
+          <t>Acend</t>
+        </is>
+      </c>
+      <c r="AV18" s="24" t="n"/>
+      <c r="AW18" s="24" t="n"/>
+      <c r="AX18" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY18" s="24" t="n"/>
+      <c r="AZ18" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA18" s="24" t="inlineStr">
+        <is>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
+        </is>
+      </c>
+      <c r="BB18" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC18" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD18" s="24" t="inlineStr">
+        <is>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
+        </is>
+      </c>
+      <c r="BE18" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF18" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG18" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH18" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T02:00:45.360175Z</t>
+        </is>
+      </c>
+      <c r="BI18" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ18" s="25" t="n"/>
+      <c r="BK18" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL18" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM18" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN18" s="28" t="n"/>
+      <c r="BO18" s="28" t="n"/>
+      <c r="BP18" s="25" t="n"/>
+      <c r="BQ18" s="27" t="n"/>
+      <c r="BR18" s="28" t="n"/>
+      <c r="BS18" s="28" t="n"/>
+      <c r="BT18" s="28" t="n"/>
+      <c r="BU18" s="25" t="n"/>
+      <c r="BV18" s="29" t="n"/>
+      <c r="BW18" s="24" t="n"/>
+      <c r="BX18" s="30" t="n"/>
+      <c r="BY18" s="27" t="n"/>
+      <c r="BZ18" s="24" t="n"/>
+      <c r="CA18" s="31" t="n"/>
+      <c r="CB18" s="24" t="n"/>
+      <c r="CC18" s="24" t="n"/>
+      <c r="CD18" s="24" t="n"/>
+      <c r="CE18" s="24" t="n"/>
+      <c r="CF18" s="24" t="n"/>
+      <c r="CG18" s="24" t="n"/>
+      <c r="CH18" s="24" t="n"/>
+      <c r="CI18" s="24" t="n"/>
+      <c r="CJ18" s="24" t="n"/>
+      <c r="CK18" s="24" t="n"/>
+      <c r="CL18" s="24" t="n"/>
+      <c r="CM18" s="24" t="n"/>
+      <c r="CN18" s="24" t="n"/>
+      <c r="CO18" s="24" t="n"/>
+      <c r="CP18" s="24" t="n"/>
+      <c r="CQ18" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>34e51feb042b446f</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T02:01:00.694416Z</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T18:30:00Z</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>71385</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>Drama eSports</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>KUUSAMO.gg</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L19" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M19" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="N19" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="O19" s="28" t="n">
+        <v>0.576412</v>
+      </c>
+      <c r="P19" s="28" t="n"/>
+      <c r="Q19" s="28" t="n">
+        <v>0.066608</v>
+      </c>
+      <c r="R19" s="26" t="n">
+        <v>53</v>
+      </c>
+      <c r="S19" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T19" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U19" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V19" s="24" t="n"/>
+      <c r="W19" s="26" t="n"/>
+      <c r="X19" s="26" t="n"/>
+      <c r="Y19" s="25" t="n"/>
+      <c r="Z19" s="26" t="n"/>
+      <c r="AA19" s="28" t="n"/>
+      <c r="AB19" s="28" t="n"/>
+      <c r="AC19" s="30" t="n"/>
+      <c r="AD19" s="24" t="n"/>
+      <c r="AE19" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5100 (market_slug=aec-cs2-ksm-drama-2026-08-04).</t>
+        </is>
+      </c>
+      <c r="AF19" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG19" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH19" s="24" t="n"/>
+      <c r="AI19" s="31" t="n"/>
+      <c r="AJ19" s="31" t="n"/>
+      <c r="AK19" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL19" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM19" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN19" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO19" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP19" s="24" t="inlineStr">
+        <is>
+          <t>Drama eSports</t>
+        </is>
+      </c>
+      <c r="AQ19" s="24" t="inlineStr">
+        <is>
+          <t>Drama eSports</t>
+        </is>
+      </c>
+      <c r="AR19" s="24" t="inlineStr">
+        <is>
+          <t>Drama eSports</t>
+        </is>
+      </c>
+      <c r="AS19" s="24" t="inlineStr">
+        <is>
+          <t>KUUSAMO.gg</t>
+        </is>
+      </c>
+      <c r="AT19" s="24" t="inlineStr">
+        <is>
+          <t>KUUSAMO.gg</t>
+        </is>
+      </c>
+      <c r="AU19" s="24" t="inlineStr">
+        <is>
+          <t>KUUSAMO.gg</t>
+        </is>
+      </c>
+      <c r="AV19" s="24" t="n"/>
+      <c r="AW19" s="24" t="n"/>
+      <c r="AX19" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY19" s="24" t="n"/>
+      <c r="AZ19" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA19" s="24" t="inlineStr">
+        <is>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
+        </is>
+      </c>
+      <c r="BB19" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC19" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD19" s="24" t="inlineStr">
+        <is>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
+        </is>
+      </c>
+      <c r="BE19" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF19" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG19" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH19" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T02:00:54.911657Z</t>
+        </is>
+      </c>
+      <c r="BI19" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ19" s="25" t="n"/>
+      <c r="BK19" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="BL19" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BM19" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="BN19" s="28" t="n"/>
+      <c r="BO19" s="28" t="n"/>
+      <c r="BP19" s="25" t="n"/>
+      <c r="BQ19" s="27" t="n"/>
+      <c r="BR19" s="28" t="n"/>
+      <c r="BS19" s="28" t="n"/>
+      <c r="BT19" s="28" t="n"/>
+      <c r="BU19" s="25" t="n"/>
+      <c r="BV19" s="29" t="n"/>
+      <c r="BW19" s="24" t="n"/>
+      <c r="BX19" s="30" t="n"/>
+      <c r="BY19" s="27" t="n"/>
+      <c r="BZ19" s="24" t="n"/>
+      <c r="CA19" s="31" t="n"/>
+      <c r="CB19" s="24" t="n"/>
+      <c r="CC19" s="24" t="n"/>
+      <c r="CD19" s="24" t="n"/>
+      <c r="CE19" s="24" t="n"/>
+      <c r="CF19" s="24" t="n"/>
+      <c r="CG19" s="24" t="n"/>
+      <c r="CH19" s="24" t="n"/>
+      <c r="CI19" s="24" t="n"/>
+      <c r="CJ19" s="24" t="n"/>
+      <c r="CK19" s="24" t="n"/>
+      <c r="CL19" s="24" t="n"/>
+      <c r="CM19" s="24" t="n"/>
+      <c r="CN19" s="24" t="n"/>
+      <c r="CO19" s="24" t="n"/>
+      <c r="CP19" s="24" t="n"/>
+      <c r="CQ19" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>bb3993ce6e8547e3</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T02:01:00.694416Z</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T18:30:00Z</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>71390</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>Subtop De France</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>Glitchtech Esports</t>
+        </is>
+      </c>
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J20" s="25" t="n"/>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L20" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M20" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="N20" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="O20" s="28" t="n">
+        <v>0.598969</v>
+      </c>
+      <c r="P20" s="28" t="n"/>
+      <c r="Q20" s="28" t="n">
+        <v>0.08916499999999999</v>
+      </c>
+      <c r="R20" s="26" t="n">
+        <v>65</v>
+      </c>
+      <c r="S20" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T20" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U20" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V20" s="24" t="n"/>
+      <c r="W20" s="26" t="n"/>
+      <c r="X20" s="26" t="n"/>
+      <c r="Y20" s="25" t="n"/>
+      <c r="Z20" s="26" t="n"/>
+      <c r="AA20" s="28" t="n"/>
+      <c r="AB20" s="28" t="n"/>
+      <c r="AC20" s="30" t="n"/>
+      <c r="AD20" s="24" t="n"/>
+      <c r="AE20" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5100 (market_slug=aec-cs2-gel-sdf-2026-08-04).</t>
+        </is>
+      </c>
+      <c r="AF20" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG20" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH20" s="24" t="n"/>
+      <c r="AI20" s="31" t="n"/>
+      <c r="AJ20" s="31" t="n"/>
+      <c r="AK20" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL20" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM20" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN20" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO20" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP20" s="24" t="inlineStr">
+        <is>
+          <t>Subtop De France</t>
+        </is>
+      </c>
+      <c r="AQ20" s="24" t="inlineStr">
+        <is>
+          <t>Subtop De France</t>
+        </is>
+      </c>
+      <c r="AR20" s="24" t="inlineStr">
+        <is>
+          <t>Subtop De France</t>
+        </is>
+      </c>
+      <c r="AS20" s="24" t="inlineStr">
+        <is>
+          <t>Glitchtech Esports</t>
+        </is>
+      </c>
+      <c r="AT20" s="24" t="inlineStr">
+        <is>
+          <t>Glitchtech Esports</t>
+        </is>
+      </c>
+      <c r="AU20" s="24" t="inlineStr">
+        <is>
+          <t>Glitchtech Esports</t>
+        </is>
+      </c>
+      <c r="AV20" s="24" t="n"/>
+      <c r="AW20" s="24" t="n"/>
+      <c r="AX20" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY20" s="24" t="n"/>
+      <c r="AZ20" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA20" s="24" t="inlineStr">
+        <is>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
+        </is>
+      </c>
+      <c r="BB20" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC20" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD20" s="24" t="inlineStr">
+        <is>
+          <t>09a1290618ceeeb656e117e9f9dc9002fa1c96576b62b6ccc86887cf39cea65f</t>
+        </is>
+      </c>
+      <c r="BE20" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF20" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG20" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH20" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T02:00:57.015430Z</t>
+        </is>
+      </c>
+      <c r="BI20" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ20" s="25" t="n"/>
+      <c r="BK20" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="BL20" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BM20" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="BN20" s="28" t="n"/>
+      <c r="BO20" s="28" t="n"/>
+      <c r="BP20" s="25" t="n"/>
+      <c r="BQ20" s="27" t="n"/>
+      <c r="BR20" s="28" t="n"/>
+      <c r="BS20" s="28" t="n"/>
+      <c r="BT20" s="28" t="n"/>
+      <c r="BU20" s="25" t="n"/>
+      <c r="BV20" s="29" t="n"/>
+      <c r="BW20" s="24" t="n"/>
+      <c r="BX20" s="30" t="n"/>
+      <c r="BY20" s="27" t="n"/>
+      <c r="BZ20" s="24" t="n"/>
+      <c r="CA20" s="31" t="n"/>
+      <c r="CB20" s="24" t="n"/>
+      <c r="CC20" s="24" t="n"/>
+      <c r="CD20" s="24" t="n"/>
+      <c r="CE20" s="24" t="n"/>
+      <c r="CF20" s="24" t="n"/>
+      <c r="CG20" s="24" t="n"/>
+      <c r="CH20" s="24" t="n"/>
+      <c r="CI20" s="24" t="n"/>
+      <c r="CJ20" s="24" t="n"/>
+      <c r="CK20" s="24" t="n"/>
+      <c r="CL20" s="24" t="n"/>
+      <c r="CM20" s="24" t="n"/>
+      <c r="CN20" s="24" t="n"/>
+      <c r="CO20" s="24" t="n"/>
+      <c r="CP20" s="24" t="n"/>
+      <c r="CQ20" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>d6d17593ded54c73</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T04:00:12.475882Z</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T18:30:00Z</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>71382</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>JUMBO TEAM</t>
+        </is>
+      </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>Benched gods</t>
+        </is>
+      </c>
+      <c r="H21" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J21" s="25" t="n"/>
+      <c r="K21" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L21" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="M21" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="N21" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="O21" s="28" t="n">
+        <v>0.67501</v>
+      </c>
+      <c r="P21" s="28" t="n"/>
+      <c r="Q21" s="28" t="n">
+        <v>0.055238</v>
+      </c>
+      <c r="R21" s="26" t="n">
+        <v>48</v>
+      </c>
+      <c r="S21" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T21" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="U21" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V21" s="24" t="n"/>
+      <c r="W21" s="26" t="n"/>
+      <c r="X21" s="26" t="n"/>
+      <c r="Y21" s="25" t="n"/>
+      <c r="Z21" s="26" t="n"/>
+      <c r="AA21" s="28" t="n"/>
+      <c r="AB21" s="28" t="n"/>
+      <c r="AC21" s="30" t="n"/>
+      <c r="AD21" s="24" t="n"/>
+      <c r="AE21" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-cs2-bge-jumbo-2026-08-04).</t>
+        </is>
+      </c>
+      <c r="AF21" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG21" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH21" s="24" t="n"/>
+      <c r="AI21" s="31" t="n"/>
+      <c r="AJ21" s="31" t="n"/>
+      <c r="AK21" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL21" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM21" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN21" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO21" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP21" s="24" t="inlineStr">
+        <is>
+          <t>JUMBO TEAM</t>
+        </is>
+      </c>
+      <c r="AQ21" s="24" t="inlineStr">
+        <is>
+          <t>JUMBO TEAM</t>
+        </is>
+      </c>
+      <c r="AR21" s="24" t="inlineStr">
+        <is>
+          <t>JUMBO TEAM</t>
+        </is>
+      </c>
+      <c r="AS21" s="24" t="inlineStr">
+        <is>
+          <t>Benched gods</t>
+        </is>
+      </c>
+      <c r="AT21" s="24" t="inlineStr">
+        <is>
+          <t>Benched gods</t>
+        </is>
+      </c>
+      <c r="AU21" s="24" t="inlineStr">
+        <is>
+          <t>Benched gods</t>
+        </is>
+      </c>
+      <c r="AV21" s="24" t="n"/>
+      <c r="AW21" s="24" t="n"/>
+      <c r="AX21" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY21" s="24" t="n"/>
+      <c r="AZ21" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA21" s="24" t="inlineStr">
+        <is>
+          <t>15c4c90af7c7e70d96e71add7b9cc8fbed98352fcea88c83a1a27ed966f78c49</t>
+        </is>
+      </c>
+      <c r="BB21" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC21" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BD21" s="24" t="inlineStr">
+        <is>
+          <t>15c4c90af7c7e70d96e71add7b9cc8fbed98352fcea88c83a1a27ed966f78c49</t>
+        </is>
+      </c>
+      <c r="BE21" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF21" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG21" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v5</t>
+        </is>
+      </c>
+      <c r="BH21" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-04T04:00:07.463015Z</t>
+        </is>
+      </c>
+      <c r="BI21" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ21" s="25" t="n"/>
+      <c r="BK21" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="BL21" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="BM21" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="BN21" s="28" t="n"/>
+      <c r="BO21" s="28" t="n"/>
+      <c r="BP21" s="25" t="n"/>
+      <c r="BQ21" s="27" t="n"/>
+      <c r="BR21" s="28" t="n"/>
+      <c r="BS21" s="28" t="n"/>
+      <c r="BT21" s="28" t="n"/>
+      <c r="BU21" s="25" t="n"/>
+      <c r="BV21" s="29" t="n"/>
+      <c r="BW21" s="24" t="n"/>
+      <c r="BX21" s="30" t="n"/>
+      <c r="BY21" s="27" t="n"/>
+      <c r="BZ21" s="24" t="n"/>
+      <c r="CA21" s="31" t="n"/>
+      <c r="CB21" s="24" t="n"/>
+      <c r="CC21" s="24" t="n"/>
+      <c r="CD21" s="24" t="n"/>
+      <c r="CE21" s="24" t="n"/>
+      <c r="CF21" s="24" t="n"/>
+      <c r="CG21" s="24" t="n"/>
+      <c r="CH21" s="24" t="n"/>
+      <c r="CI21" s="24" t="n"/>
+      <c r="CJ21" s="24" t="n"/>
+      <c r="CK21" s="24" t="n"/>
+      <c r="CL21" s="24" t="n"/>
+      <c r="CM21" s="24" t="n"/>
+      <c r="CN21" s="24" t="n"/>
+      <c r="CO21" s="24" t="n"/>
+      <c r="CP21" s="24" t="n"/>
+      <c r="CQ21" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>